<commit_message>
Update Excel Template - NG Ratio
</commit_message>
<xml_diff>
--- a/bin/Debug/Template/NGRate_Template.xlsx
+++ b/bin/Debug/Template/NGRate_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Project\My C# project\MC-Dept-App\bin\Debug\Template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Current Works\MC-Dept-App\bin\Debug\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A93E44-2596-4B5F-9286-FD405064F9C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{097E3EE0-14A0-4867-BC8E-CC92EA4FFB87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -1708,19 +1708,19 @@
     <t>Machine</t>
   </si>
   <si>
-    <t xml:space="preserve"> REF: WH-RE-006  REV:04  Date: 27/01/2025    </t>
-  </si>
-  <si>
     <t>RM Code</t>
   </si>
   <si>
     <t>Note:</t>
   </si>
   <si>
-    <t>For Account section will sign this report when each section issue dispose only.</t>
-  </si>
-  <si>
-    <t>For process transfer, return, request please follow normal process, no need acount sign.</t>
+    <t>REF: WH-RE-006  REV:05  Date: 19/03/2026</t>
+  </si>
+  <si>
+    <t>For FM/Account Section : Will sign this report only when each section issues a disposal or adjusts in/out OBS (MC-NG&amp;MC-Adjustment).</t>
+  </si>
+  <si>
+    <t>For QC Section: Will sign this report only for WH NG raw materials and NG in field processes.</t>
   </si>
 </sst>
 </file>
@@ -3750,6 +3750,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="50" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" indent="4"/>
+    </xf>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3773,96 +3776,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3939,6 +3852,96 @@
     <xf numFmtId="49" fontId="19" fillId="0" borderId="47" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -3977,96 +3980,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4143,6 +4056,96 @@
     <xf numFmtId="49" fontId="19" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4173,6 +4176,18 @@
     <xf numFmtId="0" fontId="48" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="51" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="50" fillId="4" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="50" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4197,31 +4212,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
@@ -4239,20 +4236,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="50" fillId="4" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" indent="4"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4476,8 +4476,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="154886" y="1022827"/>
-          <a:ext cx="3438516" cy="1066126"/>
+          <a:off x="154886" y="1024921"/>
+          <a:ext cx="3443749" cy="1074499"/>
           <a:chOff x="154886" y="1022575"/>
           <a:chExt cx="3435737" cy="1065086"/>
         </a:xfrm>
@@ -5237,8 +5237,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="351692" y="2224161"/>
-          <a:ext cx="1901470" cy="509712"/>
+          <a:off x="353786" y="2243001"/>
+          <a:ext cx="1904609" cy="509712"/>
           <a:chOff x="354330" y="2232660"/>
           <a:chExt cx="1901682" cy="509712"/>
         </a:xfrm>
@@ -5574,8 +5574,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="3937594" y="2224161"/>
-          <a:ext cx="2062655" cy="509712"/>
+          <a:off x="3942827" y="2243001"/>
+          <a:ext cx="2075216" cy="509712"/>
           <a:chOff x="354330" y="2232660"/>
           <a:chExt cx="1901682" cy="509712"/>
         </a:xfrm>
@@ -5911,8 +5911,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7432237" y="2043439"/>
-          <a:ext cx="2112469" cy="681097"/>
+          <a:off x="7454218" y="2051813"/>
+          <a:ext cx="2104095" cy="691563"/>
           <a:chOff x="9976701" y="1996964"/>
           <a:chExt cx="2110196" cy="682603"/>
         </a:xfrm>
@@ -6366,8 +6366,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="52551" y="4032837"/>
-          <a:ext cx="9479019" cy="1140729"/>
+          <a:off x="52551" y="4042258"/>
+          <a:ext cx="9492626" cy="1149102"/>
           <a:chOff x="52551" y="4355224"/>
           <a:chExt cx="7679120" cy="1070743"/>
         </a:xfrm>
@@ -7938,8 +7938,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="154886" y="1022827"/>
-          <a:ext cx="3438516" cy="1066126"/>
+          <a:off x="154886" y="1024921"/>
+          <a:ext cx="3443749" cy="1074499"/>
           <a:chOff x="154886" y="1022575"/>
           <a:chExt cx="3435737" cy="1065086"/>
         </a:xfrm>
@@ -8699,8 +8699,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="351692" y="2224161"/>
-          <a:ext cx="1901470" cy="509712"/>
+          <a:off x="353786" y="2243001"/>
+          <a:ext cx="1904609" cy="509712"/>
           <a:chOff x="354330" y="2232660"/>
           <a:chExt cx="1901682" cy="509712"/>
         </a:xfrm>
@@ -9036,8 +9036,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="3937594" y="2224161"/>
-          <a:ext cx="2062655" cy="509712"/>
+          <a:off x="3942827" y="2243001"/>
+          <a:ext cx="2075216" cy="509712"/>
           <a:chOff x="354330" y="2232660"/>
           <a:chExt cx="1901682" cy="509712"/>
         </a:xfrm>
@@ -9373,8 +9373,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7432237" y="2043439"/>
-          <a:ext cx="2112469" cy="681097"/>
+          <a:off x="7454218" y="2051813"/>
+          <a:ext cx="2104095" cy="691563"/>
           <a:chOff x="9976701" y="1996964"/>
           <a:chExt cx="2110196" cy="682603"/>
         </a:xfrm>
@@ -9828,8 +9828,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="52551" y="4032837"/>
-          <a:ext cx="9479019" cy="1140729"/>
+          <a:off x="52551" y="4042258"/>
+          <a:ext cx="9492626" cy="1149102"/>
           <a:chOff x="52551" y="4355224"/>
           <a:chExt cx="7679120" cy="1070743"/>
         </a:xfrm>
@@ -29034,29 +29034,29 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="26.25">
-      <c r="A3" s="320" t="s">
+      <c r="A3" s="321" t="s">
         <v>229</v>
       </c>
-      <c r="B3" s="320"/>
-      <c r="C3" s="320"/>
-      <c r="D3" s="320"/>
-      <c r="E3" s="320"/>
-      <c r="F3" s="320"/>
-      <c r="G3" s="320"/>
-      <c r="H3" s="320"/>
-      <c r="I3" s="320"/>
-      <c r="J3" s="320"/>
-      <c r="K3" s="320"/>
-      <c r="L3" s="320"/>
+      <c r="B3" s="321"/>
+      <c r="C3" s="321"/>
+      <c r="D3" s="321"/>
+      <c r="E3" s="321"/>
+      <c r="F3" s="321"/>
+      <c r="G3" s="321"/>
+      <c r="H3" s="321"/>
+      <c r="I3" s="321"/>
+      <c r="J3" s="321"/>
+      <c r="K3" s="321"/>
+      <c r="L3" s="321"/>
     </row>
     <row r="4" spans="1:12" ht="20.100000000000001" customHeight="1">
       <c r="H4" s="56" t="s">
         <v>88</v>
       </c>
-      <c r="I4" s="389">
+      <c r="I4" s="390">
         <v>45390</v>
       </c>
-      <c r="J4" s="389"/>
+      <c r="J4" s="390"/>
       <c r="K4" s="73"/>
       <c r="L4" s="73"/>
     </row>
@@ -29070,12 +29070,12 @@
       <c r="H5" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="I5" s="326" t="s">
+      <c r="I5" s="327" t="s">
         <v>418</v>
       </c>
-      <c r="J5" s="326"/>
-      <c r="K5" s="326"/>
-      <c r="L5" s="326"/>
+      <c r="J5" s="327"/>
+      <c r="K5" s="327"/>
+      <c r="L5" s="327"/>
     </row>
     <row r="6" spans="1:12" ht="20.25" customHeight="1">
       <c r="B6" t="s">
@@ -29084,10 +29084,10 @@
       <c r="H6" s="56" t="s">
         <v>90</v>
       </c>
-      <c r="I6" s="326" t="s">
+      <c r="I6" s="327" t="s">
         <v>419</v>
       </c>
-      <c r="J6" s="326"/>
+      <c r="J6" s="327"/>
       <c r="K6" s="74"/>
       <c r="L6" s="74"/>
     </row>
@@ -29118,32 +29118,32 @@
       <c r="L8" s="13"/>
     </row>
     <row r="9" spans="1:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="J9" s="327" t="s">
+      <c r="J9" s="328" t="s">
         <v>132</v>
       </c>
-      <c r="K9" s="328" t="s">
+      <c r="K9" s="329" t="s">
         <v>140</v>
       </c>
-      <c r="L9" s="329"/>
+      <c r="L9" s="330"/>
     </row>
     <row r="10" spans="1:12">
       <c r="B10" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="323" t="s">
+      <c r="C10" s="324" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="324"/>
-      <c r="E10" s="325"/>
+      <c r="D10" s="325"/>
+      <c r="E10" s="326"/>
       <c r="F10" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="G10" s="323" t="s">
+      <c r="G10" s="324" t="s">
         <v>56</v>
       </c>
-      <c r="H10" s="324"/>
+      <c r="H10" s="325"/>
       <c r="I10" s="13"/>
-      <c r="J10" s="327"/>
+      <c r="J10" s="328"/>
       <c r="K10" s="9" t="s">
         <v>141</v>
       </c>
@@ -29155,14 +29155,14 @@
       <c r="B11" s="221" t="s">
         <v>417</v>
       </c>
-      <c r="C11" s="387" t="s">
+      <c r="C11" s="388" t="s">
         <v>69</v>
       </c>
-      <c r="D11" s="388"/>
-      <c r="E11" s="325"/>
+      <c r="D11" s="389"/>
+      <c r="E11" s="326"/>
       <c r="F11" s="51"/>
-      <c r="G11" s="321"/>
-      <c r="H11" s="322"/>
+      <c r="G11" s="322"/>
+      <c r="H11" s="323"/>
       <c r="I11" s="13"/>
       <c r="J11" s="9"/>
       <c r="K11" s="10"/>
@@ -29928,10 +29928,10 @@
       <c r="L33" s="9"/>
     </row>
     <row r="34" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A34" s="390" t="s">
+      <c r="A34" s="391" t="s">
         <v>392</v>
       </c>
-      <c r="B34" s="390"/>
+      <c r="B34" s="391"/>
       <c r="C34" s="67"/>
       <c r="D34" s="222"/>
       <c r="E34" s="219"/>
@@ -29948,27 +29948,27 @@
     </row>
     <row r="35" spans="1:12" ht="13.5" customHeight="1"/>
     <row r="36" spans="1:12">
-      <c r="A36" s="328" t="s">
+      <c r="A36" s="329" t="s">
         <v>95</v>
       </c>
-      <c r="B36" s="329"/>
-      <c r="C36" s="393" t="s">
+      <c r="B36" s="330"/>
+      <c r="C36" s="394" t="s">
         <v>93</v>
       </c>
-      <c r="D36" s="394"/>
-      <c r="E36" s="328" t="s">
+      <c r="D36" s="395"/>
+      <c r="E36" s="329" t="s">
         <v>221</v>
       </c>
-      <c r="F36" s="329"/>
-      <c r="G36" s="327" t="s">
+      <c r="F36" s="330"/>
+      <c r="G36" s="328" t="s">
         <v>231</v>
       </c>
-      <c r="H36" s="327"/>
-      <c r="I36" s="327"/>
-      <c r="J36" s="391" t="s">
+      <c r="H36" s="328"/>
+      <c r="I36" s="328"/>
+      <c r="J36" s="392" t="s">
         <v>230</v>
       </c>
-      <c r="K36" s="392"/>
+      <c r="K36" s="393"/>
     </row>
     <row r="37" spans="1:12">
       <c r="A37" s="65"/>
@@ -30029,11 +30029,11 @@
         <v>88</v>
       </c>
       <c r="F41" s="68"/>
-      <c r="G41" s="317" t="s">
+      <c r="G41" s="318" t="s">
         <v>88</v>
       </c>
-      <c r="H41" s="318"/>
-      <c r="I41" s="319"/>
+      <c r="H41" s="319"/>
+      <c r="I41" s="320"/>
       <c r="J41" s="67" t="s">
         <v>88</v>
       </c>
@@ -30041,16 +30041,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="G41:I41"/>
     <mergeCell ref="J36:K36"/>
     <mergeCell ref="C11:D11"/>
@@ -30060,6 +30050,16 @@
     <mergeCell ref="C36:D36"/>
     <mergeCell ref="E36:F36"/>
     <mergeCell ref="G36:I36"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="G10:H10"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="70" orientation="portrait" r:id="rId1"/>
@@ -30094,7 +30094,7 @@
         <v>142</v>
       </c>
       <c r="J1" s="228" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75">
@@ -30103,28 +30103,28 @@
       </c>
     </row>
     <row r="3" spans="1:13" ht="25.5">
-      <c r="A3" s="403" t="s">
+      <c r="A3" s="397" t="s">
         <v>229</v>
       </c>
-      <c r="B3" s="403"/>
-      <c r="C3" s="403"/>
-      <c r="D3" s="403"/>
-      <c r="E3" s="403"/>
-      <c r="F3" s="403"/>
-      <c r="G3" s="403"/>
-      <c r="H3" s="403"/>
-      <c r="I3" s="403"/>
-      <c r="J3" s="403"/>
-      <c r="K3" s="403"/>
-      <c r="L3" s="403"/>
-      <c r="M3" s="403"/>
+      <c r="B3" s="397"/>
+      <c r="C3" s="397"/>
+      <c r="D3" s="397"/>
+      <c r="E3" s="397"/>
+      <c r="F3" s="397"/>
+      <c r="G3" s="397"/>
+      <c r="H3" s="397"/>
+      <c r="I3" s="397"/>
+      <c r="J3" s="397"/>
+      <c r="K3" s="397"/>
+      <c r="L3" s="397"/>
+      <c r="M3" s="397"/>
     </row>
     <row r="4" spans="1:13" ht="20.100000000000001" customHeight="1">
       <c r="I4" s="230" t="s">
         <v>88</v>
       </c>
-      <c r="J4" s="420"/>
-      <c r="K4" s="420"/>
+      <c r="J4" s="398"/>
+      <c r="K4" s="398"/>
       <c r="L4" s="231"/>
       <c r="M4" s="231"/>
     </row>
@@ -30132,21 +30132,21 @@
       <c r="I5" s="230" t="s">
         <v>89</v>
       </c>
-      <c r="J5" s="404" t="s">
+      <c r="J5" s="399" t="s">
         <v>423</v>
       </c>
-      <c r="K5" s="404"/>
-      <c r="L5" s="405"/>
-      <c r="M5" s="405"/>
+      <c r="K5" s="399"/>
+      <c r="L5" s="396"/>
+      <c r="M5" s="396"/>
     </row>
     <row r="6" spans="1:13" ht="20.25" customHeight="1">
       <c r="I6" s="230" t="s">
         <v>90</v>
       </c>
-      <c r="J6" s="404" t="s">
+      <c r="J6" s="399" t="s">
         <v>424</v>
       </c>
-      <c r="K6" s="404"/>
+      <c r="K6" s="399"/>
       <c r="L6" s="232"/>
       <c r="M6" s="232"/>
     </row>
@@ -30154,13 +30154,13 @@
       <c r="I7" s="230" t="s">
         <v>91</v>
       </c>
-      <c r="J7" s="405"/>
-      <c r="K7" s="405"/>
-      <c r="L7" s="405"/>
+      <c r="J7" s="396"/>
+      <c r="K7" s="396"/>
+      <c r="L7" s="396"/>
       <c r="M7" s="232"/>
     </row>
     <row r="8" spans="1:13" ht="20.25" customHeight="1">
-      <c r="E8" s="421"/>
+      <c r="E8" s="254"/>
       <c r="I8" s="233"/>
       <c r="J8" s="234"/>
       <c r="K8" s="234"/>
@@ -30168,33 +30168,33 @@
       <c r="M8" s="234"/>
     </row>
     <row r="9" spans="1:13" ht="13.5" customHeight="1">
-      <c r="K9" s="401"/>
-      <c r="L9" s="402"/>
-      <c r="M9" s="402"/>
+      <c r="K9" s="406"/>
+      <c r="L9" s="407"/>
+      <c r="M9" s="407"/>
     </row>
     <row r="10" spans="1:13">
       <c r="B10" s="234"/>
-      <c r="C10" s="402"/>
-      <c r="D10" s="402"/>
-      <c r="E10" s="401"/>
+      <c r="C10" s="407"/>
+      <c r="D10" s="407"/>
+      <c r="E10" s="406"/>
       <c r="F10" s="235"/>
       <c r="G10" s="234"/>
-      <c r="H10" s="402"/>
-      <c r="I10" s="402"/>
+      <c r="H10" s="407"/>
+      <c r="I10" s="407"/>
       <c r="J10" s="234"/>
-      <c r="K10" s="401"/>
+      <c r="K10" s="406"/>
       <c r="L10" s="234"/>
       <c r="M10" s="236"/>
     </row>
     <row r="11" spans="1:13" ht="26.25" customHeight="1">
       <c r="B11" s="235"/>
-      <c r="C11" s="401"/>
-      <c r="D11" s="401"/>
-      <c r="E11" s="401"/>
+      <c r="C11" s="406"/>
+      <c r="D11" s="406"/>
+      <c r="E11" s="406"/>
       <c r="F11" s="235"/>
       <c r="G11" s="235"/>
-      <c r="H11" s="401"/>
-      <c r="I11" s="401"/>
+      <c r="H11" s="406"/>
+      <c r="I11" s="406"/>
       <c r="J11" s="234"/>
       <c r="K11" s="234"/>
     </row>
@@ -30210,12 +30210,12 @@
         <v>225</v>
       </c>
       <c r="D13" s="238" t="s">
-        <v>426</v>
-      </c>
-      <c r="E13" s="395" t="s">
+        <v>425</v>
+      </c>
+      <c r="E13" s="400" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="396"/>
+      <c r="F13" s="401"/>
       <c r="G13" s="238" t="s">
         <v>52</v>
       </c>
@@ -30243,8 +30243,8 @@
       <c r="B14" s="239"/>
       <c r="C14" s="239"/>
       <c r="D14" s="240"/>
-      <c r="E14" s="397"/>
-      <c r="F14" s="398"/>
+      <c r="E14" s="402"/>
+      <c r="F14" s="403"/>
       <c r="G14" s="241"/>
       <c r="H14" s="242"/>
       <c r="I14" s="243"/>
@@ -30254,12 +30254,12 @@
       <c r="M14" s="247"/>
     </row>
     <row r="15" spans="1:13" ht="16.5" customHeight="1">
-      <c r="A15" s="399" t="s">
+      <c r="A15" s="404" t="s">
         <v>392</v>
       </c>
-      <c r="B15" s="400"/>
-      <c r="C15" s="400"/>
-      <c r="D15" s="400"/>
+      <c r="B15" s="405"/>
+      <c r="C15" s="405"/>
+      <c r="D15" s="405"/>
       <c r="E15" s="248"/>
       <c r="F15" s="248"/>
       <c r="G15" s="248"/>
@@ -30276,7 +30276,7 @@
     <row r="16" spans="1:13" ht="13.5" customHeight="1"/>
     <row r="26" spans="4:5">
       <c r="D26" s="252" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E26" s="253" t="s">
         <v>428</v>
@@ -30290,12 +30290,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="J6:K6"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="A15:D15"/>
@@ -30306,6 +30300,12 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="J6:K6"/>
   </mergeCells>
   <pageMargins left="0.1" right="0.1" top="0.2" bottom="0.2" header="0.1" footer="0.1"/>
   <pageSetup paperSize="9" scale="71" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -30341,7 +30341,7 @@
         <v>142</v>
       </c>
       <c r="J1" s="228" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75">
@@ -30350,28 +30350,28 @@
       </c>
     </row>
     <row r="3" spans="1:13" ht="25.5">
-      <c r="A3" s="403" t="s">
+      <c r="A3" s="397" t="s">
         <v>229</v>
       </c>
-      <c r="B3" s="403"/>
-      <c r="C3" s="403"/>
-      <c r="D3" s="403"/>
-      <c r="E3" s="403"/>
-      <c r="F3" s="403"/>
-      <c r="G3" s="403"/>
-      <c r="H3" s="403"/>
-      <c r="I3" s="403"/>
-      <c r="J3" s="403"/>
-      <c r="K3" s="403"/>
-      <c r="L3" s="403"/>
-      <c r="M3" s="403"/>
+      <c r="B3" s="397"/>
+      <c r="C3" s="397"/>
+      <c r="D3" s="397"/>
+      <c r="E3" s="397"/>
+      <c r="F3" s="397"/>
+      <c r="G3" s="397"/>
+      <c r="H3" s="397"/>
+      <c r="I3" s="397"/>
+      <c r="J3" s="397"/>
+      <c r="K3" s="397"/>
+      <c r="L3" s="397"/>
+      <c r="M3" s="397"/>
     </row>
     <row r="4" spans="1:13" ht="20.100000000000001" customHeight="1">
       <c r="I4" s="230" t="s">
         <v>88</v>
       </c>
-      <c r="J4" s="420"/>
-      <c r="K4" s="420"/>
+      <c r="J4" s="398"/>
+      <c r="K4" s="398"/>
       <c r="L4" s="231"/>
       <c r="M4" s="231"/>
     </row>
@@ -30379,21 +30379,21 @@
       <c r="I5" s="230" t="s">
         <v>89</v>
       </c>
-      <c r="J5" s="404" t="s">
+      <c r="J5" s="399" t="s">
         <v>423</v>
       </c>
-      <c r="K5" s="404"/>
-      <c r="L5" s="405"/>
-      <c r="M5" s="405"/>
+      <c r="K5" s="399"/>
+      <c r="L5" s="396"/>
+      <c r="M5" s="396"/>
     </row>
     <row r="6" spans="1:13" ht="20.25" customHeight="1">
       <c r="I6" s="230" t="s">
         <v>90</v>
       </c>
-      <c r="J6" s="404" t="s">
+      <c r="J6" s="399" t="s">
         <v>424</v>
       </c>
-      <c r="K6" s="404"/>
+      <c r="K6" s="399"/>
       <c r="L6" s="232"/>
       <c r="M6" s="232"/>
     </row>
@@ -30401,13 +30401,13 @@
       <c r="I7" s="230" t="s">
         <v>91</v>
       </c>
-      <c r="J7" s="405"/>
-      <c r="K7" s="405"/>
-      <c r="L7" s="405"/>
+      <c r="J7" s="396"/>
+      <c r="K7" s="396"/>
+      <c r="L7" s="396"/>
       <c r="M7" s="232"/>
     </row>
     <row r="8" spans="1:13" ht="20.25" customHeight="1">
-      <c r="E8" s="421"/>
+      <c r="E8" s="254"/>
       <c r="I8" s="233"/>
       <c r="J8" s="234"/>
       <c r="K8" s="234"/>
@@ -30415,33 +30415,33 @@
       <c r="M8" s="234"/>
     </row>
     <row r="9" spans="1:13" ht="13.5" customHeight="1">
-      <c r="K9" s="401"/>
-      <c r="L9" s="402"/>
-      <c r="M9" s="402"/>
+      <c r="K9" s="406"/>
+      <c r="L9" s="407"/>
+      <c r="M9" s="407"/>
     </row>
     <row r="10" spans="1:13">
       <c r="B10" s="234"/>
-      <c r="C10" s="402"/>
-      <c r="D10" s="402"/>
-      <c r="E10" s="401"/>
+      <c r="C10" s="407"/>
+      <c r="D10" s="407"/>
+      <c r="E10" s="406"/>
       <c r="F10" s="235"/>
       <c r="G10" s="234"/>
-      <c r="H10" s="402"/>
-      <c r="I10" s="402"/>
+      <c r="H10" s="407"/>
+      <c r="I10" s="407"/>
       <c r="J10" s="234"/>
-      <c r="K10" s="401"/>
+      <c r="K10" s="406"/>
       <c r="L10" s="234"/>
       <c r="M10" s="236"/>
     </row>
     <row r="11" spans="1:13" ht="26.25" customHeight="1">
       <c r="B11" s="235"/>
-      <c r="C11" s="401"/>
-      <c r="D11" s="401"/>
-      <c r="E11" s="401"/>
+      <c r="C11" s="406"/>
+      <c r="D11" s="406"/>
+      <c r="E11" s="406"/>
       <c r="F11" s="235"/>
       <c r="G11" s="235"/>
-      <c r="H11" s="401"/>
-      <c r="I11" s="401"/>
+      <c r="H11" s="406"/>
+      <c r="I11" s="406"/>
       <c r="J11" s="234"/>
       <c r="K11" s="234"/>
     </row>
@@ -30457,12 +30457,12 @@
         <v>225</v>
       </c>
       <c r="D13" s="238" t="s">
-        <v>426</v>
-      </c>
-      <c r="E13" s="395" t="s">
+        <v>425</v>
+      </c>
+      <c r="E13" s="400" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="396"/>
+      <c r="F13" s="401"/>
       <c r="G13" s="238" t="s">
         <v>52</v>
       </c>
@@ -30490,8 +30490,8 @@
       <c r="B14" s="239"/>
       <c r="C14" s="239"/>
       <c r="D14" s="240"/>
-      <c r="E14" s="397"/>
-      <c r="F14" s="398"/>
+      <c r="E14" s="402"/>
+      <c r="F14" s="403"/>
       <c r="G14" s="241"/>
       <c r="H14" s="242"/>
       <c r="I14" s="243"/>
@@ -30501,12 +30501,12 @@
       <c r="M14" s="247"/>
     </row>
     <row r="15" spans="1:13" ht="16.5" customHeight="1">
-      <c r="A15" s="399" t="s">
+      <c r="A15" s="404" t="s">
         <v>392</v>
       </c>
-      <c r="B15" s="400"/>
-      <c r="C15" s="400"/>
-      <c r="D15" s="400"/>
+      <c r="B15" s="405"/>
+      <c r="C15" s="405"/>
+      <c r="D15" s="405"/>
       <c r="E15" s="248"/>
       <c r="F15" s="248"/>
       <c r="G15" s="248"/>
@@ -30523,7 +30523,7 @@
     <row r="16" spans="1:13" ht="13.5" customHeight="1"/>
     <row r="26" spans="4:5">
       <c r="D26" s="252" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E26" s="253" t="s">
         <v>428</v>
@@ -30537,6 +30537,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="J6:K6"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="A15:D15"/>
@@ -30547,12 +30553,6 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="H11:I11"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="J7:L7"/>
   </mergeCells>
   <pageMargins left="0.1" right="0.1" top="0.2" bottom="0.2" header="0.1" footer="0.1"/>
   <pageSetup paperSize="9" scale="71" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -30591,32 +30591,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="417" t="s">
+      <c r="A1" s="408" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="417"/>
-      <c r="C1" s="417"/>
-      <c r="D1" s="417"/>
-      <c r="E1" s="417"/>
-      <c r="F1" s="417"/>
-      <c r="G1" s="417"/>
-      <c r="H1" s="417"/>
-      <c r="I1" s="417"/>
-      <c r="J1" s="417"/>
+      <c r="B1" s="408"/>
+      <c r="C1" s="408"/>
+      <c r="D1" s="408"/>
+      <c r="E1" s="408"/>
+      <c r="F1" s="408"/>
+      <c r="G1" s="408"/>
+      <c r="H1" s="408"/>
+      <c r="I1" s="408"/>
+      <c r="J1" s="408"/>
     </row>
     <row r="2" spans="1:10" ht="26.25">
-      <c r="A2" s="320" t="s">
+      <c r="A2" s="321" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="320"/>
-      <c r="C2" s="320"/>
-      <c r="D2" s="320"/>
-      <c r="E2" s="320"/>
-      <c r="F2" s="320"/>
-      <c r="G2" s="320"/>
-      <c r="H2" s="320"/>
-      <c r="I2" s="320"/>
-      <c r="J2" s="320"/>
+      <c r="B2" s="321"/>
+      <c r="C2" s="321"/>
+      <c r="D2" s="321"/>
+      <c r="E2" s="321"/>
+      <c r="F2" s="321"/>
+      <c r="G2" s="321"/>
+      <c r="H2" s="321"/>
+      <c r="I2" s="321"/>
+      <c r="J2" s="321"/>
     </row>
     <row r="3" spans="1:10" ht="20.25" customHeight="1">
       <c r="H3" s="56" t="s">
@@ -30632,8 +30632,8 @@
       <c r="H4" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="I4" s="326"/>
-      <c r="J4" s="326"/>
+      <c r="I4" s="327"/>
+      <c r="J4" s="327"/>
     </row>
     <row r="5" spans="1:10" ht="20.25" customHeight="1">
       <c r="B5" t="s">
@@ -30677,11 +30677,11 @@
       <c r="B10" s="53" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="418" t="s">
+      <c r="C10" s="409" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="418"/>
-      <c r="E10" s="418"/>
+      <c r="D10" s="409"/>
+      <c r="E10" s="409"/>
       <c r="F10" s="53" t="s">
         <v>52</v>
       </c>
@@ -30691,442 +30691,442 @@
       <c r="H10" s="53" t="s">
         <v>54</v>
       </c>
-      <c r="I10" s="418" t="s">
+      <c r="I10" s="409" t="s">
         <v>6</v>
       </c>
-      <c r="J10" s="419"/>
+      <c r="J10" s="410"/>
     </row>
     <row r="11" spans="1:10" ht="20.25" customHeight="1" thickTop="1">
       <c r="A11" s="69">
         <v>1</v>
       </c>
       <c r="B11" s="6"/>
-      <c r="C11" s="412"/>
-      <c r="D11" s="413"/>
-      <c r="E11" s="414"/>
+      <c r="C11" s="411"/>
+      <c r="D11" s="412"/>
+      <c r="E11" s="413"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
-      <c r="I11" s="415"/>
-      <c r="J11" s="416"/>
+      <c r="I11" s="414"/>
+      <c r="J11" s="415"/>
     </row>
     <row r="12" spans="1:10" ht="20.25" customHeight="1">
       <c r="A12" s="70">
         <v>2</v>
       </c>
       <c r="B12" s="10"/>
-      <c r="C12" s="317"/>
-      <c r="D12" s="318"/>
-      <c r="E12" s="319"/>
+      <c r="C12" s="318"/>
+      <c r="D12" s="319"/>
+      <c r="E12" s="320"/>
       <c r="F12" s="10"/>
       <c r="G12" s="10"/>
       <c r="H12" s="10"/>
-      <c r="I12" s="328"/>
-      <c r="J12" s="411"/>
+      <c r="I12" s="329"/>
+      <c r="J12" s="416"/>
     </row>
     <row r="13" spans="1:10" ht="20.25" customHeight="1">
       <c r="A13" s="69">
         <v>3</v>
       </c>
       <c r="B13" s="10"/>
-      <c r="C13" s="317"/>
-      <c r="D13" s="318"/>
-      <c r="E13" s="319"/>
+      <c r="C13" s="318"/>
+      <c r="D13" s="319"/>
+      <c r="E13" s="320"/>
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
       <c r="H13" s="10"/>
-      <c r="I13" s="328"/>
-      <c r="J13" s="411"/>
+      <c r="I13" s="329"/>
+      <c r="J13" s="416"/>
     </row>
     <row r="14" spans="1:10" ht="20.25" customHeight="1">
       <c r="A14" s="70">
         <v>4</v>
       </c>
       <c r="B14" s="10"/>
-      <c r="C14" s="317"/>
-      <c r="D14" s="318"/>
-      <c r="E14" s="319"/>
+      <c r="C14" s="318"/>
+      <c r="D14" s="319"/>
+      <c r="E14" s="320"/>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
       <c r="H14" s="10"/>
-      <c r="I14" s="328"/>
-      <c r="J14" s="411"/>
+      <c r="I14" s="329"/>
+      <c r="J14" s="416"/>
     </row>
     <row r="15" spans="1:10" ht="20.25" customHeight="1">
       <c r="A15" s="69">
         <v>5</v>
       </c>
       <c r="B15" s="10"/>
-      <c r="C15" s="317"/>
-      <c r="D15" s="318"/>
-      <c r="E15" s="319"/>
+      <c r="C15" s="318"/>
+      <c r="D15" s="319"/>
+      <c r="E15" s="320"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="10"/>
-      <c r="I15" s="328"/>
-      <c r="J15" s="411"/>
+      <c r="I15" s="329"/>
+      <c r="J15" s="416"/>
     </row>
     <row r="16" spans="1:10" ht="20.25" customHeight="1">
       <c r="A16" s="70">
         <v>6</v>
       </c>
       <c r="B16" s="10"/>
-      <c r="C16" s="317"/>
-      <c r="D16" s="318"/>
-      <c r="E16" s="319"/>
+      <c r="C16" s="318"/>
+      <c r="D16" s="319"/>
+      <c r="E16" s="320"/>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
       <c r="H16" s="10"/>
-      <c r="I16" s="328"/>
-      <c r="J16" s="411"/>
+      <c r="I16" s="329"/>
+      <c r="J16" s="416"/>
     </row>
     <row r="17" spans="1:10" ht="20.25" customHeight="1">
       <c r="A17" s="69">
         <v>7</v>
       </c>
       <c r="B17" s="10"/>
-      <c r="C17" s="317"/>
-      <c r="D17" s="318"/>
-      <c r="E17" s="319"/>
+      <c r="C17" s="318"/>
+      <c r="D17" s="319"/>
+      <c r="E17" s="320"/>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
-      <c r="I17" s="328"/>
-      <c r="J17" s="411"/>
+      <c r="I17" s="329"/>
+      <c r="J17" s="416"/>
     </row>
     <row r="18" spans="1:10" ht="20.25" customHeight="1">
       <c r="A18" s="70">
         <v>8</v>
       </c>
       <c r="B18" s="10"/>
-      <c r="C18" s="317"/>
-      <c r="D18" s="318"/>
-      <c r="E18" s="319"/>
+      <c r="C18" s="318"/>
+      <c r="D18" s="319"/>
+      <c r="E18" s="320"/>
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
       <c r="H18" s="10"/>
-      <c r="I18" s="328"/>
-      <c r="J18" s="411"/>
+      <c r="I18" s="329"/>
+      <c r="J18" s="416"/>
     </row>
     <row r="19" spans="1:10" ht="20.25" customHeight="1">
       <c r="A19" s="69">
         <v>9</v>
       </c>
       <c r="B19" s="10"/>
-      <c r="C19" s="317"/>
-      <c r="D19" s="318"/>
-      <c r="E19" s="319"/>
+      <c r="C19" s="318"/>
+      <c r="D19" s="319"/>
+      <c r="E19" s="320"/>
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
       <c r="H19" s="10"/>
-      <c r="I19" s="328"/>
-      <c r="J19" s="411"/>
+      <c r="I19" s="329"/>
+      <c r="J19" s="416"/>
     </row>
     <row r="20" spans="1:10" ht="20.25" customHeight="1">
       <c r="A20" s="70">
         <v>10</v>
       </c>
       <c r="B20" s="10"/>
-      <c r="C20" s="317"/>
-      <c r="D20" s="318"/>
-      <c r="E20" s="319"/>
+      <c r="C20" s="318"/>
+      <c r="D20" s="319"/>
+      <c r="E20" s="320"/>
       <c r="F20" s="10"/>
       <c r="G20" s="10"/>
       <c r="H20" s="10"/>
-      <c r="I20" s="328"/>
-      <c r="J20" s="411"/>
+      <c r="I20" s="329"/>
+      <c r="J20" s="416"/>
     </row>
     <row r="21" spans="1:10" ht="20.25" customHeight="1">
       <c r="A21" s="69">
         <v>11</v>
       </c>
       <c r="B21" s="10"/>
-      <c r="C21" s="317"/>
-      <c r="D21" s="318"/>
-      <c r="E21" s="319"/>
+      <c r="C21" s="318"/>
+      <c r="D21" s="319"/>
+      <c r="E21" s="320"/>
       <c r="F21" s="10"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
-      <c r="I21" s="328"/>
-      <c r="J21" s="411"/>
+      <c r="I21" s="329"/>
+      <c r="J21" s="416"/>
     </row>
     <row r="22" spans="1:10" ht="20.25" customHeight="1">
       <c r="A22" s="70">
         <v>12</v>
       </c>
       <c r="B22" s="10"/>
-      <c r="C22" s="317"/>
-      <c r="D22" s="318"/>
-      <c r="E22" s="319"/>
+      <c r="C22" s="318"/>
+      <c r="D22" s="319"/>
+      <c r="E22" s="320"/>
       <c r="F22" s="10"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
-      <c r="I22" s="328"/>
-      <c r="J22" s="411"/>
+      <c r="I22" s="329"/>
+      <c r="J22" s="416"/>
     </row>
     <row r="23" spans="1:10" ht="20.25" customHeight="1">
       <c r="A23" s="69">
         <v>13</v>
       </c>
       <c r="B23" s="10"/>
-      <c r="C23" s="317"/>
-      <c r="D23" s="318"/>
-      <c r="E23" s="319"/>
+      <c r="C23" s="318"/>
+      <c r="D23" s="319"/>
+      <c r="E23" s="320"/>
       <c r="F23" s="10"/>
       <c r="G23" s="10"/>
       <c r="H23" s="10"/>
-      <c r="I23" s="328"/>
-      <c r="J23" s="411"/>
+      <c r="I23" s="329"/>
+      <c r="J23" s="416"/>
     </row>
     <row r="24" spans="1:10" ht="20.25" customHeight="1">
       <c r="A24" s="70">
         <v>14</v>
       </c>
       <c r="B24" s="10"/>
-      <c r="C24" s="317"/>
-      <c r="D24" s="318"/>
-      <c r="E24" s="319"/>
+      <c r="C24" s="318"/>
+      <c r="D24" s="319"/>
+      <c r="E24" s="320"/>
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10"/>
-      <c r="I24" s="328"/>
-      <c r="J24" s="411"/>
+      <c r="I24" s="329"/>
+      <c r="J24" s="416"/>
     </row>
     <row r="25" spans="1:10" ht="20.25" customHeight="1">
       <c r="A25" s="69">
         <v>15</v>
       </c>
       <c r="B25" s="10"/>
-      <c r="C25" s="317"/>
-      <c r="D25" s="318"/>
-      <c r="E25" s="319"/>
+      <c r="C25" s="318"/>
+      <c r="D25" s="319"/>
+      <c r="E25" s="320"/>
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
       <c r="H25" s="10"/>
-      <c r="I25" s="328"/>
-      <c r="J25" s="411"/>
+      <c r="I25" s="329"/>
+      <c r="J25" s="416"/>
     </row>
     <row r="26" spans="1:10" ht="20.25" customHeight="1">
       <c r="A26" s="70">
         <v>16</v>
       </c>
       <c r="B26" s="10"/>
-      <c r="C26" s="317"/>
-      <c r="D26" s="318"/>
-      <c r="E26" s="319"/>
+      <c r="C26" s="318"/>
+      <c r="D26" s="319"/>
+      <c r="E26" s="320"/>
       <c r="F26" s="10"/>
       <c r="G26" s="10"/>
       <c r="H26" s="10"/>
-      <c r="I26" s="328"/>
-      <c r="J26" s="411"/>
+      <c r="I26" s="329"/>
+      <c r="J26" s="416"/>
     </row>
     <row r="27" spans="1:10" ht="20.25" customHeight="1">
       <c r="A27" s="69">
         <v>17</v>
       </c>
       <c r="B27" s="10"/>
-      <c r="C27" s="317"/>
-      <c r="D27" s="318"/>
-      <c r="E27" s="319"/>
+      <c r="C27" s="318"/>
+      <c r="D27" s="319"/>
+      <c r="E27" s="320"/>
       <c r="F27" s="10"/>
       <c r="G27" s="10"/>
       <c r="H27" s="10"/>
-      <c r="I27" s="328"/>
-      <c r="J27" s="411"/>
+      <c r="I27" s="329"/>
+      <c r="J27" s="416"/>
     </row>
     <row r="28" spans="1:10" ht="20.25" customHeight="1">
       <c r="A28" s="70">
         <v>18</v>
       </c>
       <c r="B28" s="10"/>
-      <c r="C28" s="317"/>
-      <c r="D28" s="318"/>
-      <c r="E28" s="319"/>
+      <c r="C28" s="318"/>
+      <c r="D28" s="319"/>
+      <c r="E28" s="320"/>
       <c r="F28" s="10"/>
       <c r="G28" s="10"/>
       <c r="H28" s="10"/>
-      <c r="I28" s="328"/>
-      <c r="J28" s="411"/>
+      <c r="I28" s="329"/>
+      <c r="J28" s="416"/>
     </row>
     <row r="29" spans="1:10" ht="20.25" customHeight="1">
       <c r="A29" s="69">
         <v>19</v>
       </c>
       <c r="B29" s="10"/>
-      <c r="C29" s="317"/>
-      <c r="D29" s="318"/>
-      <c r="E29" s="319"/>
+      <c r="C29" s="318"/>
+      <c r="D29" s="319"/>
+      <c r="E29" s="320"/>
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
       <c r="H29" s="10"/>
-      <c r="I29" s="328"/>
-      <c r="J29" s="411"/>
+      <c r="I29" s="329"/>
+      <c r="J29" s="416"/>
     </row>
     <row r="30" spans="1:10" ht="20.25" customHeight="1">
       <c r="A30" s="70">
         <v>20</v>
       </c>
       <c r="B30" s="10"/>
-      <c r="C30" s="317"/>
-      <c r="D30" s="318"/>
-      <c r="E30" s="319"/>
+      <c r="C30" s="318"/>
+      <c r="D30" s="319"/>
+      <c r="E30" s="320"/>
       <c r="F30" s="10"/>
       <c r="G30" s="10"/>
       <c r="H30" s="10"/>
-      <c r="I30" s="328"/>
-      <c r="J30" s="411"/>
+      <c r="I30" s="329"/>
+      <c r="J30" s="416"/>
     </row>
     <row r="31" spans="1:10" ht="20.25" customHeight="1">
       <c r="A31" s="69">
         <v>21</v>
       </c>
       <c r="B31" s="10"/>
-      <c r="C31" s="317"/>
-      <c r="D31" s="318"/>
-      <c r="E31" s="319"/>
+      <c r="C31" s="318"/>
+      <c r="D31" s="319"/>
+      <c r="E31" s="320"/>
       <c r="F31" s="10"/>
       <c r="G31" s="10"/>
       <c r="H31" s="10"/>
-      <c r="I31" s="328"/>
-      <c r="J31" s="411"/>
+      <c r="I31" s="329"/>
+      <c r="J31" s="416"/>
     </row>
     <row r="32" spans="1:10" ht="20.25" customHeight="1">
       <c r="A32" s="70">
         <v>22</v>
       </c>
       <c r="B32" s="10"/>
-      <c r="C32" s="317"/>
-      <c r="D32" s="318"/>
-      <c r="E32" s="319"/>
+      <c r="C32" s="318"/>
+      <c r="D32" s="319"/>
+      <c r="E32" s="320"/>
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
       <c r="H32" s="10"/>
-      <c r="I32" s="328"/>
-      <c r="J32" s="411"/>
+      <c r="I32" s="329"/>
+      <c r="J32" s="416"/>
     </row>
     <row r="33" spans="1:10" ht="20.25" customHeight="1">
       <c r="A33" s="69">
         <v>23</v>
       </c>
       <c r="B33" s="10"/>
-      <c r="C33" s="317"/>
-      <c r="D33" s="318"/>
-      <c r="E33" s="319"/>
+      <c r="C33" s="318"/>
+      <c r="D33" s="319"/>
+      <c r="E33" s="320"/>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
       <c r="H33" s="10"/>
-      <c r="I33" s="328"/>
-      <c r="J33" s="411"/>
+      <c r="I33" s="329"/>
+      <c r="J33" s="416"/>
     </row>
     <row r="34" spans="1:10" ht="20.25" customHeight="1">
       <c r="A34" s="70">
         <v>24</v>
       </c>
       <c r="B34" s="10"/>
-      <c r="C34" s="317"/>
-      <c r="D34" s="318"/>
-      <c r="E34" s="319"/>
+      <c r="C34" s="318"/>
+      <c r="D34" s="319"/>
+      <c r="E34" s="320"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
       <c r="H34" s="10"/>
-      <c r="I34" s="328"/>
-      <c r="J34" s="411"/>
+      <c r="I34" s="329"/>
+      <c r="J34" s="416"/>
     </row>
     <row r="35" spans="1:10" ht="20.25" customHeight="1">
       <c r="A35" s="69">
         <v>25</v>
       </c>
       <c r="B35" s="10"/>
-      <c r="C35" s="317"/>
-      <c r="D35" s="318"/>
-      <c r="E35" s="319"/>
+      <c r="C35" s="318"/>
+      <c r="D35" s="319"/>
+      <c r="E35" s="320"/>
       <c r="F35" s="10"/>
       <c r="G35" s="10"/>
       <c r="H35" s="10"/>
-      <c r="I35" s="328"/>
-      <c r="J35" s="411"/>
+      <c r="I35" s="329"/>
+      <c r="J35" s="416"/>
     </row>
     <row r="36" spans="1:10" ht="20.25" customHeight="1">
       <c r="A36" s="69">
         <v>26</v>
       </c>
       <c r="B36" s="71"/>
-      <c r="C36" s="317"/>
-      <c r="D36" s="318"/>
-      <c r="E36" s="319"/>
+      <c r="C36" s="318"/>
+      <c r="D36" s="319"/>
+      <c r="E36" s="320"/>
       <c r="F36" s="71"/>
       <c r="G36" s="71"/>
       <c r="H36" s="71"/>
-      <c r="I36" s="328"/>
-      <c r="J36" s="411"/>
+      <c r="I36" s="329"/>
+      <c r="J36" s="416"/>
     </row>
     <row r="37" spans="1:10" ht="20.25" customHeight="1">
       <c r="A37" s="69">
         <v>27</v>
       </c>
       <c r="B37" s="71"/>
-      <c r="C37" s="317"/>
-      <c r="D37" s="318"/>
-      <c r="E37" s="319"/>
+      <c r="C37" s="318"/>
+      <c r="D37" s="319"/>
+      <c r="E37" s="320"/>
       <c r="F37" s="71"/>
       <c r="G37" s="71"/>
       <c r="H37" s="71"/>
-      <c r="I37" s="328"/>
-      <c r="J37" s="411"/>
+      <c r="I37" s="329"/>
+      <c r="J37" s="416"/>
     </row>
     <row r="38" spans="1:10" ht="20.25" customHeight="1">
       <c r="A38" s="69">
         <v>28</v>
       </c>
       <c r="B38" s="71"/>
-      <c r="C38" s="317"/>
-      <c r="D38" s="318"/>
-      <c r="E38" s="319"/>
+      <c r="C38" s="318"/>
+      <c r="D38" s="319"/>
+      <c r="E38" s="320"/>
       <c r="F38" s="71"/>
       <c r="G38" s="71"/>
       <c r="H38" s="71"/>
-      <c r="I38" s="328"/>
-      <c r="J38" s="411"/>
+      <c r="I38" s="329"/>
+      <c r="J38" s="416"/>
     </row>
     <row r="39" spans="1:10" ht="20.25" customHeight="1">
       <c r="A39" s="69">
         <v>29</v>
       </c>
       <c r="B39" s="71"/>
-      <c r="C39" s="317"/>
-      <c r="D39" s="318"/>
-      <c r="E39" s="319"/>
+      <c r="C39" s="318"/>
+      <c r="D39" s="319"/>
+      <c r="E39" s="320"/>
       <c r="F39" s="71"/>
       <c r="G39" s="71"/>
       <c r="H39" s="71"/>
-      <c r="I39" s="328"/>
-      <c r="J39" s="411"/>
+      <c r="I39" s="329"/>
+      <c r="J39" s="416"/>
     </row>
     <row r="40" spans="1:10" ht="20.25" customHeight="1">
       <c r="A40" s="69">
         <v>30</v>
       </c>
       <c r="B40" s="71"/>
-      <c r="C40" s="317"/>
-      <c r="D40" s="318"/>
-      <c r="E40" s="319"/>
+      <c r="C40" s="318"/>
+      <c r="D40" s="319"/>
+      <c r="E40" s="320"/>
       <c r="F40" s="71"/>
       <c r="G40" s="71"/>
       <c r="H40" s="71"/>
-      <c r="I40" s="328"/>
-      <c r="J40" s="411"/>
+      <c r="I40" s="329"/>
+      <c r="J40" s="416"/>
     </row>
     <row r="41" spans="1:10" ht="8.25" customHeight="1" thickBot="1">
       <c r="A41" s="54"/>
       <c r="B41" s="55"/>
-      <c r="C41" s="406"/>
-      <c r="D41" s="407"/>
-      <c r="E41" s="408"/>
+      <c r="C41" s="417"/>
+      <c r="D41" s="418"/>
+      <c r="E41" s="419"/>
       <c r="F41" s="55"/>
       <c r="G41" s="55"/>
       <c r="H41" s="55"/>
-      <c r="I41" s="409"/>
-      <c r="J41" s="410"/>
+      <c r="I41" s="420"/>
+      <c r="J41" s="421"/>
     </row>
     <row r="42" spans="1:10" ht="14.25" customHeight="1">
       <c r="C42" s="72"/>
@@ -31143,26 +31143,26 @@
       <c r="J43" s="13"/>
     </row>
     <row r="45" spans="1:10">
-      <c r="A45" s="328" t="s">
+      <c r="A45" s="329" t="s">
         <v>95</v>
       </c>
-      <c r="B45" s="329"/>
-      <c r="C45" s="328" t="s">
+      <c r="B45" s="330"/>
+      <c r="C45" s="329" t="s">
         <v>94</v>
       </c>
-      <c r="D45" s="329"/>
-      <c r="E45" s="328" t="s">
+      <c r="D45" s="330"/>
+      <c r="E45" s="329" t="s">
         <v>93</v>
       </c>
-      <c r="F45" s="329"/>
-      <c r="G45" s="328" t="s">
+      <c r="F45" s="330"/>
+      <c r="G45" s="329" t="s">
         <v>114</v>
       </c>
-      <c r="H45" s="329"/>
-      <c r="I45" s="328" t="s">
+      <c r="H45" s="330"/>
+      <c r="I45" s="329" t="s">
         <v>92</v>
       </c>
-      <c r="J45" s="329"/>
+      <c r="J45" s="330"/>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="65"/>
@@ -31236,71 +31236,6 @@
     </row>
   </sheetData>
   <mergeCells count="72">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="I40:J40"/>
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="I41:J41"/>
     <mergeCell ref="A45:B45"/>
@@ -31308,6 +31243,71 @@
     <mergeCell ref="E45:F45"/>
     <mergeCell ref="G45:H45"/>
     <mergeCell ref="I45:J45"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="I10:J10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -31939,52 +31939,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="31.7" customHeight="1">
-      <c r="A1" s="254" t="s">
+      <c r="A1" s="255" t="s">
         <v>170</v>
       </c>
-      <c r="B1" s="254"/>
-      <c r="C1" s="254"/>
-      <c r="D1" s="254"/>
-      <c r="E1" s="254"/>
-      <c r="F1" s="254"/>
-      <c r="G1" s="254"/>
-      <c r="H1" s="254"/>
-      <c r="I1" s="254"/>
-      <c r="J1" s="254"/>
-      <c r="K1" s="254"/>
-      <c r="L1" s="254"/>
-      <c r="M1" s="254"/>
-      <c r="N1" s="254"/>
-      <c r="O1" s="254"/>
-      <c r="P1" s="254"/>
-      <c r="Q1" s="254"/>
+      <c r="B1" s="255"/>
+      <c r="C1" s="255"/>
+      <c r="D1" s="255"/>
+      <c r="E1" s="255"/>
+      <c r="F1" s="255"/>
+      <c r="G1" s="255"/>
+      <c r="H1" s="255"/>
+      <c r="I1" s="255"/>
+      <c r="J1" s="255"/>
+      <c r="K1" s="255"/>
+      <c r="L1" s="255"/>
+      <c r="M1" s="255"/>
+      <c r="N1" s="255"/>
+      <c r="O1" s="255"/>
+      <c r="P1" s="255"/>
+      <c r="Q1" s="255"/>
     </row>
     <row r="2" spans="1:17" s="77" customFormat="1" ht="23.45" customHeight="1">
-      <c r="A2" s="255" t="s">
+      <c r="A2" s="256" t="s">
         <v>171</v>
       </c>
-      <c r="B2" s="255"/>
-      <c r="C2" s="255"/>
-      <c r="D2" s="255"/>
-      <c r="E2" s="255"/>
-      <c r="F2" s="255"/>
-      <c r="G2" s="256" t="s">
+      <c r="B2" s="256"/>
+      <c r="C2" s="256"/>
+      <c r="D2" s="256"/>
+      <c r="E2" s="256"/>
+      <c r="F2" s="256"/>
+      <c r="G2" s="257" t="s">
         <v>98</v>
       </c>
-      <c r="H2" s="256"/>
-      <c r="I2" s="256"/>
-      <c r="J2" s="256"/>
-      <c r="K2" s="256"/>
-      <c r="L2" s="256"/>
-      <c r="M2" s="257" t="s">
+      <c r="H2" s="257"/>
+      <c r="I2" s="257"/>
+      <c r="J2" s="257"/>
+      <c r="K2" s="257"/>
+      <c r="L2" s="257"/>
+      <c r="M2" s="258" t="s">
         <v>172</v>
       </c>
-      <c r="N2" s="258" t="s">
+      <c r="N2" s="259" t="s">
         <v>173</v>
       </c>
-      <c r="O2" s="259"/>
-      <c r="P2" s="259"/>
-      <c r="Q2" s="260"/>
+      <c r="O2" s="260"/>
+      <c r="P2" s="260"/>
+      <c r="Q2" s="261"/>
     </row>
     <row r="3" spans="1:17" ht="30">
       <c r="A3" s="136"/>
@@ -31996,14 +31996,14 @@
       <c r="G3" s="139" t="s">
         <v>96</v>
       </c>
-      <c r="H3" s="261" t="s">
+      <c r="H3" s="262" t="s">
         <v>174</v>
       </c>
-      <c r="I3" s="261"/>
-      <c r="J3" s="261"/>
-      <c r="K3" s="261"/>
-      <c r="L3" s="261"/>
-      <c r="M3" s="257"/>
+      <c r="I3" s="262"/>
+      <c r="J3" s="262"/>
+      <c r="K3" s="262"/>
+      <c r="L3" s="262"/>
+      <c r="M3" s="258"/>
       <c r="N3" s="140" t="s">
         <v>175</v>
       </c>
@@ -34067,152 +34067,152 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="20.25" customHeight="1">
-      <c r="A1" s="262" t="s">
+      <c r="A1" s="300" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="263"/>
-      <c r="C1" s="263"/>
-      <c r="D1" s="263"/>
-      <c r="E1" s="263"/>
-      <c r="F1" s="263"/>
-      <c r="G1" s="263"/>
-      <c r="H1" s="264"/>
-      <c r="I1" s="265" t="s">
+      <c r="B1" s="301"/>
+      <c r="C1" s="301"/>
+      <c r="D1" s="301"/>
+      <c r="E1" s="301"/>
+      <c r="F1" s="301"/>
+      <c r="G1" s="301"/>
+      <c r="H1" s="302"/>
+      <c r="I1" s="303" t="s">
         <v>143</v>
       </c>
-      <c r="J1" s="266"/>
-      <c r="K1" s="267"/>
-      <c r="L1" s="268" t="s">
+      <c r="J1" s="304"/>
+      <c r="K1" s="305"/>
+      <c r="L1" s="306" t="s">
         <v>144</v>
       </c>
-      <c r="M1" s="269"/>
-      <c r="N1" s="270"/>
+      <c r="M1" s="307"/>
+      <c r="N1" s="308"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1">
-      <c r="A2" s="271" t="s">
+      <c r="A2" s="309" t="s">
         <v>145</v>
       </c>
-      <c r="B2" s="272"/>
-      <c r="C2" s="272"/>
-      <c r="D2" s="272"/>
-      <c r="E2" s="272"/>
-      <c r="F2" s="272"/>
-      <c r="G2" s="272"/>
-      <c r="H2" s="273"/>
-      <c r="I2" s="274" t="s">
+      <c r="B2" s="310"/>
+      <c r="C2" s="310"/>
+      <c r="D2" s="310"/>
+      <c r="E2" s="310"/>
+      <c r="F2" s="310"/>
+      <c r="G2" s="310"/>
+      <c r="H2" s="311"/>
+      <c r="I2" s="312" t="s">
         <v>146</v>
       </c>
-      <c r="J2" s="275"/>
-      <c r="K2" s="276"/>
-      <c r="L2" s="277" t="s">
+      <c r="J2" s="313"/>
+      <c r="K2" s="314"/>
+      <c r="L2" s="315" t="s">
         <v>147</v>
       </c>
-      <c r="M2" s="278"/>
-      <c r="N2" s="279"/>
+      <c r="M2" s="316"/>
+      <c r="N2" s="317"/>
     </row>
     <row r="3" spans="1:14" ht="30.75" customHeight="1">
-      <c r="A3" s="280" t="s">
+      <c r="A3" s="288" t="s">
         <v>148</v>
       </c>
-      <c r="B3" s="281"/>
-      <c r="C3" s="281"/>
-      <c r="D3" s="281"/>
-      <c r="E3" s="281"/>
-      <c r="F3" s="281"/>
-      <c r="G3" s="281"/>
-      <c r="H3" s="282"/>
-      <c r="I3" s="283" t="s">
+      <c r="B3" s="289"/>
+      <c r="C3" s="289"/>
+      <c r="D3" s="289"/>
+      <c r="E3" s="289"/>
+      <c r="F3" s="289"/>
+      <c r="G3" s="289"/>
+      <c r="H3" s="290"/>
+      <c r="I3" s="291" t="s">
         <v>149</v>
       </c>
-      <c r="J3" s="284"/>
-      <c r="K3" s="283" t="s">
+      <c r="J3" s="292"/>
+      <c r="K3" s="291" t="s">
         <v>150</v>
       </c>
-      <c r="L3" s="284"/>
-      <c r="M3" s="283" t="s">
+      <c r="L3" s="292"/>
+      <c r="M3" s="291" t="s">
         <v>151</v>
       </c>
-      <c r="N3" s="285"/>
+      <c r="N3" s="293"/>
     </row>
     <row r="4" spans="1:14" ht="43.5" customHeight="1">
       <c r="A4" s="85" t="s">
         <v>152</v>
       </c>
-      <c r="B4" s="286" t="s">
+      <c r="B4" s="294" t="s">
         <v>153</v>
       </c>
-      <c r="C4" s="287"/>
-      <c r="D4" s="287"/>
-      <c r="E4" s="287"/>
-      <c r="F4" s="287"/>
-      <c r="G4" s="287"/>
-      <c r="H4" s="288"/>
-      <c r="I4" s="289"/>
-      <c r="J4" s="290"/>
-      <c r="K4" s="289"/>
-      <c r="L4" s="290"/>
-      <c r="M4" s="289"/>
-      <c r="N4" s="291"/>
+      <c r="C4" s="295"/>
+      <c r="D4" s="295"/>
+      <c r="E4" s="295"/>
+      <c r="F4" s="295"/>
+      <c r="G4" s="295"/>
+      <c r="H4" s="296"/>
+      <c r="I4" s="297"/>
+      <c r="J4" s="298"/>
+      <c r="K4" s="297"/>
+      <c r="L4" s="298"/>
+      <c r="M4" s="297"/>
+      <c r="N4" s="299"/>
     </row>
     <row r="5" spans="1:14" s="87" customFormat="1" ht="46.5" customHeight="1">
       <c r="A5" s="86">
         <v>1</v>
       </c>
-      <c r="B5" s="294" t="s">
+      <c r="B5" s="265" t="s">
         <v>154</v>
       </c>
-      <c r="C5" s="295"/>
-      <c r="D5" s="295"/>
-      <c r="E5" s="295"/>
-      <c r="F5" s="295"/>
-      <c r="G5" s="295"/>
-      <c r="H5" s="295"/>
-      <c r="I5" s="295"/>
-      <c r="J5" s="295"/>
-      <c r="K5" s="295"/>
-      <c r="L5" s="295"/>
-      <c r="M5" s="295"/>
-      <c r="N5" s="296"/>
+      <c r="C5" s="266"/>
+      <c r="D5" s="266"/>
+      <c r="E5" s="266"/>
+      <c r="F5" s="266"/>
+      <c r="G5" s="266"/>
+      <c r="H5" s="266"/>
+      <c r="I5" s="266"/>
+      <c r="J5" s="266"/>
+      <c r="K5" s="266"/>
+      <c r="L5" s="266"/>
+      <c r="M5" s="266"/>
+      <c r="N5" s="267"/>
     </row>
     <row r="6" spans="1:14" s="87" customFormat="1" ht="39" customHeight="1">
       <c r="A6" s="88">
         <v>2</v>
       </c>
-      <c r="B6" s="297" t="s">
+      <c r="B6" s="268" t="s">
         <v>155</v>
       </c>
-      <c r="C6" s="298"/>
-      <c r="D6" s="298"/>
-      <c r="E6" s="298"/>
-      <c r="F6" s="298"/>
-      <c r="G6" s="298"/>
-      <c r="H6" s="298"/>
-      <c r="I6" s="298"/>
-      <c r="J6" s="298"/>
-      <c r="K6" s="298"/>
-      <c r="L6" s="298"/>
-      <c r="M6" s="298"/>
-      <c r="N6" s="299"/>
+      <c r="C6" s="269"/>
+      <c r="D6" s="269"/>
+      <c r="E6" s="269"/>
+      <c r="F6" s="269"/>
+      <c r="G6" s="269"/>
+      <c r="H6" s="269"/>
+      <c r="I6" s="269"/>
+      <c r="J6" s="269"/>
+      <c r="K6" s="269"/>
+      <c r="L6" s="269"/>
+      <c r="M6" s="269"/>
+      <c r="N6" s="270"/>
     </row>
     <row r="7" spans="1:14" s="87" customFormat="1" ht="21" customHeight="1">
       <c r="A7" s="89" t="s">
         <v>156</v>
       </c>
-      <c r="B7" s="300" t="s">
+      <c r="B7" s="271" t="s">
         <v>157</v>
       </c>
-      <c r="C7" s="301"/>
-      <c r="D7" s="301"/>
-      <c r="E7" s="301"/>
-      <c r="F7" s="301"/>
-      <c r="G7" s="301"/>
-      <c r="H7" s="301"/>
-      <c r="I7" s="301"/>
-      <c r="J7" s="301"/>
-      <c r="K7" s="301"/>
-      <c r="L7" s="301"/>
-      <c r="M7" s="301"/>
-      <c r="N7" s="302"/>
+      <c r="C7" s="272"/>
+      <c r="D7" s="272"/>
+      <c r="E7" s="272"/>
+      <c r="F7" s="272"/>
+      <c r="G7" s="272"/>
+      <c r="H7" s="272"/>
+      <c r="I7" s="272"/>
+      <c r="J7" s="272"/>
+      <c r="K7" s="272"/>
+      <c r="L7" s="272"/>
+      <c r="M7" s="272"/>
+      <c r="N7" s="273"/>
     </row>
     <row r="8" spans="1:14" s="95" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="90"/>
@@ -34781,7 +34781,7 @@
       <c r="N42" s="99"/>
     </row>
     <row r="43" spans="1:14" s="123" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A43" s="303" t="s">
+      <c r="A43" s="274" t="s">
         <v>162</v>
       </c>
       <c r="B43" s="116" t="s">
@@ -34789,81 +34789,95 @@
       </c>
       <c r="C43" s="117"/>
       <c r="D43" s="118"/>
-      <c r="E43" s="306"/>
-      <c r="F43" s="307"/>
-      <c r="G43" s="307"/>
-      <c r="H43" s="307"/>
-      <c r="I43" s="307"/>
-      <c r="J43" s="307"/>
+      <c r="E43" s="277"/>
+      <c r="F43" s="278"/>
+      <c r="G43" s="278"/>
+      <c r="H43" s="278"/>
+      <c r="I43" s="278"/>
+      <c r="J43" s="278"/>
       <c r="K43" s="121"/>
       <c r="L43" s="120"/>
       <c r="M43" s="119"/>
       <c r="N43" s="122"/>
     </row>
     <row r="44" spans="1:14" s="123" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A44" s="304"/>
+      <c r="A44" s="275"/>
       <c r="B44" s="124" t="s">
         <v>163</v>
       </c>
       <c r="C44" s="125"/>
       <c r="D44" s="126"/>
-      <c r="E44" s="308"/>
-      <c r="F44" s="309"/>
-      <c r="G44" s="309"/>
-      <c r="H44" s="309"/>
-      <c r="I44" s="309"/>
-      <c r="J44" s="309"/>
+      <c r="E44" s="279"/>
+      <c r="F44" s="280"/>
+      <c r="G44" s="280"/>
+      <c r="H44" s="280"/>
+      <c r="I44" s="280"/>
+      <c r="J44" s="280"/>
       <c r="K44" s="127"/>
       <c r="L44" s="128"/>
       <c r="M44" s="129"/>
       <c r="N44" s="130"/>
     </row>
     <row r="45" spans="1:14" s="123" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A45" s="304"/>
+      <c r="A45" s="275"/>
       <c r="B45" s="131" t="s">
         <v>164</v>
       </c>
       <c r="C45" s="125"/>
       <c r="D45" s="126"/>
-      <c r="E45" s="310"/>
-      <c r="F45" s="311"/>
-      <c r="G45" s="311"/>
-      <c r="H45" s="311"/>
-      <c r="I45" s="311"/>
-      <c r="J45" s="311"/>
+      <c r="E45" s="281"/>
+      <c r="F45" s="282"/>
+      <c r="G45" s="282"/>
+      <c r="H45" s="282"/>
+      <c r="I45" s="282"/>
+      <c r="J45" s="282"/>
       <c r="K45" s="132"/>
       <c r="L45" s="128"/>
       <c r="M45" s="133"/>
       <c r="N45" s="134"/>
     </row>
     <row r="46" spans="1:14" s="123" customFormat="1" ht="25.5" customHeight="1" thickBot="1">
-      <c r="A46" s="305"/>
+      <c r="A46" s="276"/>
       <c r="B46" s="135" t="s">
         <v>165</v>
       </c>
-      <c r="C46" s="312" t="s">
+      <c r="C46" s="283" t="s">
         <v>166</v>
       </c>
-      <c r="D46" s="313"/>
-      <c r="E46" s="314" t="s">
+      <c r="D46" s="284"/>
+      <c r="E46" s="285" t="s">
         <v>167</v>
       </c>
-      <c r="F46" s="315"/>
-      <c r="G46" s="315"/>
-      <c r="H46" s="315"/>
-      <c r="I46" s="315"/>
-      <c r="J46" s="316"/>
-      <c r="K46" s="292" t="s">
+      <c r="F46" s="286"/>
+      <c r="G46" s="286"/>
+      <c r="H46" s="286"/>
+      <c r="I46" s="286"/>
+      <c r="J46" s="287"/>
+      <c r="K46" s="263" t="s">
         <v>168</v>
       </c>
-      <c r="L46" s="316"/>
-      <c r="M46" s="292" t="s">
+      <c r="L46" s="287"/>
+      <c r="M46" s="263" t="s">
         <v>169</v>
       </c>
-      <c r="N46" s="293"/>
+      <c r="N46" s="264"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="M46:N46"/>
     <mergeCell ref="B5:N5"/>
     <mergeCell ref="B6:N6"/>
@@ -34875,20 +34889,6 @@
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="E46:J46"/>
     <mergeCell ref="K46:L46"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="L2:N2"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -34931,20 +34931,20 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="26.25">
-      <c r="A3" s="320" t="s">
+      <c r="A3" s="321" t="s">
         <v>229</v>
       </c>
-      <c r="B3" s="320"/>
-      <c r="C3" s="320"/>
-      <c r="D3" s="320"/>
-      <c r="E3" s="320"/>
-      <c r="F3" s="320"/>
-      <c r="G3" s="320"/>
-      <c r="H3" s="320"/>
-      <c r="I3" s="320"/>
-      <c r="J3" s="320"/>
-      <c r="K3" s="320"/>
-      <c r="L3" s="320"/>
+      <c r="B3" s="321"/>
+      <c r="C3" s="321"/>
+      <c r="D3" s="321"/>
+      <c r="E3" s="321"/>
+      <c r="F3" s="321"/>
+      <c r="G3" s="321"/>
+      <c r="H3" s="321"/>
+      <c r="I3" s="321"/>
+      <c r="J3" s="321"/>
+      <c r="K3" s="321"/>
+      <c r="L3" s="321"/>
     </row>
     <row r="4" spans="1:12" ht="20.100000000000001" customHeight="1">
       <c r="H4" s="56" t="s">
@@ -34965,10 +34965,10 @@
       <c r="H5" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="I5" s="326"/>
-      <c r="J5" s="326"/>
-      <c r="K5" s="326"/>
-      <c r="L5" s="326"/>
+      <c r="I5" s="327"/>
+      <c r="J5" s="327"/>
+      <c r="K5" s="327"/>
+      <c r="L5" s="327"/>
     </row>
     <row r="6" spans="1:12" ht="20.25" customHeight="1">
       <c r="B6" t="s">
@@ -35007,32 +35007,32 @@
       <c r="L8" s="13"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1">
-      <c r="J9" s="327" t="s">
+      <c r="J9" s="328" t="s">
         <v>132</v>
       </c>
-      <c r="K9" s="328" t="s">
+      <c r="K9" s="329" t="s">
         <v>140</v>
       </c>
-      <c r="L9" s="329"/>
+      <c r="L9" s="330"/>
     </row>
     <row r="10" spans="1:12">
       <c r="B10" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="323" t="s">
+      <c r="C10" s="324" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="324"/>
-      <c r="E10" s="325"/>
+      <c r="D10" s="325"/>
+      <c r="E10" s="326"/>
       <c r="F10" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="G10" s="323" t="s">
+      <c r="G10" s="324" t="s">
         <v>56</v>
       </c>
-      <c r="H10" s="324"/>
+      <c r="H10" s="325"/>
       <c r="I10" s="13"/>
-      <c r="J10" s="327"/>
+      <c r="J10" s="328"/>
       <c r="K10" s="9" t="s">
         <v>141</v>
       </c>
@@ -35042,12 +35042,12 @@
     </row>
     <row r="11" spans="1:12" ht="26.25" customHeight="1" thickBot="1">
       <c r="B11" s="51"/>
-      <c r="C11" s="321"/>
-      <c r="D11" s="322"/>
-      <c r="E11" s="325"/>
+      <c r="C11" s="322"/>
+      <c r="D11" s="323"/>
+      <c r="E11" s="326"/>
       <c r="F11" s="51"/>
-      <c r="G11" s="321"/>
-      <c r="H11" s="322"/>
+      <c r="G11" s="322"/>
+      <c r="H11" s="323"/>
       <c r="I11" s="13"/>
       <c r="J11" s="9"/>
       <c r="K11" s="10"/>
@@ -35730,23 +35730,23 @@
       <c r="L54" s="13"/>
     </row>
     <row r="56" spans="1:12">
-      <c r="A56" s="328" t="s">
+      <c r="A56" s="329" t="s">
         <v>95</v>
       </c>
-      <c r="B56" s="329"/>
-      <c r="C56" s="328" t="s">
+      <c r="B56" s="330"/>
+      <c r="C56" s="329" t="s">
         <v>93</v>
       </c>
-      <c r="D56" s="329"/>
-      <c r="E56" s="328" t="s">
+      <c r="D56" s="330"/>
+      <c r="E56" s="329" t="s">
         <v>221</v>
       </c>
-      <c r="F56" s="329"/>
-      <c r="G56" s="327" t="s">
+      <c r="F56" s="330"/>
+      <c r="G56" s="328" t="s">
         <v>231</v>
       </c>
-      <c r="H56" s="327"/>
-      <c r="I56" s="327"/>
+      <c r="H56" s="328"/>
+      <c r="I56" s="328"/>
       <c r="J56" s="58" t="s">
         <v>230</v>
       </c>
@@ -35806,11 +35806,11 @@
         <v>88</v>
       </c>
       <c r="F61" s="68"/>
-      <c r="G61" s="317" t="s">
+      <c r="G61" s="318" t="s">
         <v>88</v>
       </c>
-      <c r="H61" s="318"/>
-      <c r="I61" s="319"/>
+      <c r="H61" s="319"/>
+      <c r="I61" s="320"/>
       <c r="J61" s="10" t="s">
         <v>88</v>
       </c>
@@ -35853,52 +35853,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="31.7" customHeight="1">
-      <c r="A1" s="254" t="s">
+      <c r="A1" s="255" t="s">
         <v>170</v>
       </c>
-      <c r="B1" s="254"/>
-      <c r="C1" s="254"/>
-      <c r="D1" s="254"/>
-      <c r="E1" s="254"/>
-      <c r="F1" s="254"/>
-      <c r="G1" s="254"/>
-      <c r="H1" s="254"/>
-      <c r="I1" s="254"/>
-      <c r="J1" s="254"/>
-      <c r="K1" s="254"/>
-      <c r="L1" s="254"/>
-      <c r="M1" s="254"/>
-      <c r="N1" s="254"/>
-      <c r="O1" s="254"/>
-      <c r="P1" s="254"/>
-      <c r="Q1" s="254"/>
+      <c r="B1" s="255"/>
+      <c r="C1" s="255"/>
+      <c r="D1" s="255"/>
+      <c r="E1" s="255"/>
+      <c r="F1" s="255"/>
+      <c r="G1" s="255"/>
+      <c r="H1" s="255"/>
+      <c r="I1" s="255"/>
+      <c r="J1" s="255"/>
+      <c r="K1" s="255"/>
+      <c r="L1" s="255"/>
+      <c r="M1" s="255"/>
+      <c r="N1" s="255"/>
+      <c r="O1" s="255"/>
+      <c r="P1" s="255"/>
+      <c r="Q1" s="255"/>
     </row>
     <row r="2" spans="1:17" s="77" customFormat="1" ht="23.45" customHeight="1">
-      <c r="A2" s="255" t="s">
+      <c r="A2" s="256" t="s">
         <v>171</v>
       </c>
-      <c r="B2" s="255"/>
-      <c r="C2" s="255"/>
-      <c r="D2" s="255"/>
-      <c r="E2" s="255"/>
-      <c r="F2" s="255"/>
-      <c r="G2" s="255" t="s">
+      <c r="B2" s="256"/>
+      <c r="C2" s="256"/>
+      <c r="D2" s="256"/>
+      <c r="E2" s="256"/>
+      <c r="F2" s="256"/>
+      <c r="G2" s="256" t="s">
         <v>98</v>
       </c>
-      <c r="H2" s="255"/>
-      <c r="I2" s="255"/>
-      <c r="J2" s="255"/>
-      <c r="K2" s="255"/>
-      <c r="L2" s="255"/>
-      <c r="M2" s="257" t="s">
+      <c r="H2" s="256"/>
+      <c r="I2" s="256"/>
+      <c r="J2" s="256"/>
+      <c r="K2" s="256"/>
+      <c r="L2" s="256"/>
+      <c r="M2" s="258" t="s">
         <v>172</v>
       </c>
-      <c r="N2" s="258" t="s">
+      <c r="N2" s="259" t="s">
         <v>173</v>
       </c>
-      <c r="O2" s="259"/>
-      <c r="P2" s="259"/>
-      <c r="Q2" s="260"/>
+      <c r="O2" s="260"/>
+      <c r="P2" s="260"/>
+      <c r="Q2" s="261"/>
     </row>
     <row r="3" spans="1:17" ht="30">
       <c r="A3" s="136"/>
@@ -35910,14 +35910,14 @@
       <c r="G3" s="139" t="s">
         <v>96</v>
       </c>
-      <c r="H3" s="261" t="s">
+      <c r="H3" s="262" t="s">
         <v>174</v>
       </c>
-      <c r="I3" s="261"/>
-      <c r="J3" s="261"/>
-      <c r="K3" s="261"/>
-      <c r="L3" s="261"/>
-      <c r="M3" s="257"/>
+      <c r="I3" s="262"/>
+      <c r="J3" s="262"/>
+      <c r="K3" s="262"/>
+      <c r="L3" s="262"/>
+      <c r="M3" s="258"/>
       <c r="N3" s="140" t="s">
         <v>175</v>
       </c>
@@ -38134,152 +38134,152 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="20.25" customHeight="1">
-      <c r="A1" s="330" t="s">
+      <c r="A1" s="368" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="331"/>
-      <c r="C1" s="331"/>
-      <c r="D1" s="331"/>
-      <c r="E1" s="331"/>
-      <c r="F1" s="331"/>
-      <c r="G1" s="331"/>
-      <c r="H1" s="332"/>
-      <c r="I1" s="333" t="s">
+      <c r="B1" s="369"/>
+      <c r="C1" s="369"/>
+      <c r="D1" s="369"/>
+      <c r="E1" s="369"/>
+      <c r="F1" s="369"/>
+      <c r="G1" s="369"/>
+      <c r="H1" s="370"/>
+      <c r="I1" s="371" t="s">
         <v>143</v>
       </c>
-      <c r="J1" s="334"/>
-      <c r="K1" s="335"/>
-      <c r="L1" s="336" t="s">
+      <c r="J1" s="372"/>
+      <c r="K1" s="373"/>
+      <c r="L1" s="374" t="s">
         <v>144</v>
       </c>
-      <c r="M1" s="337"/>
-      <c r="N1" s="338"/>
+      <c r="M1" s="375"/>
+      <c r="N1" s="376"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1">
-      <c r="A2" s="339" t="s">
+      <c r="A2" s="377" t="s">
         <v>145</v>
       </c>
-      <c r="B2" s="340"/>
-      <c r="C2" s="340"/>
-      <c r="D2" s="340"/>
-      <c r="E2" s="340"/>
-      <c r="F2" s="340"/>
-      <c r="G2" s="340"/>
-      <c r="H2" s="341"/>
-      <c r="I2" s="342" t="s">
+      <c r="B2" s="378"/>
+      <c r="C2" s="378"/>
+      <c r="D2" s="378"/>
+      <c r="E2" s="378"/>
+      <c r="F2" s="378"/>
+      <c r="G2" s="378"/>
+      <c r="H2" s="379"/>
+      <c r="I2" s="380" t="s">
         <v>146</v>
       </c>
-      <c r="J2" s="343"/>
-      <c r="K2" s="344"/>
-      <c r="L2" s="345" t="s">
+      <c r="J2" s="381"/>
+      <c r="K2" s="382"/>
+      <c r="L2" s="383" t="s">
         <v>147</v>
       </c>
-      <c r="M2" s="346"/>
-      <c r="N2" s="347"/>
+      <c r="M2" s="384"/>
+      <c r="N2" s="385"/>
     </row>
     <row r="3" spans="1:14" ht="30.75" customHeight="1">
-      <c r="A3" s="348" t="s">
+      <c r="A3" s="356" t="s">
         <v>148</v>
       </c>
-      <c r="B3" s="349"/>
-      <c r="C3" s="349"/>
-      <c r="D3" s="349"/>
-      <c r="E3" s="349"/>
-      <c r="F3" s="349"/>
-      <c r="G3" s="349"/>
-      <c r="H3" s="350"/>
-      <c r="I3" s="351" t="s">
+      <c r="B3" s="357"/>
+      <c r="C3" s="357"/>
+      <c r="D3" s="357"/>
+      <c r="E3" s="357"/>
+      <c r="F3" s="357"/>
+      <c r="G3" s="357"/>
+      <c r="H3" s="358"/>
+      <c r="I3" s="359" t="s">
         <v>149</v>
       </c>
-      <c r="J3" s="352"/>
-      <c r="K3" s="351" t="s">
+      <c r="J3" s="360"/>
+      <c r="K3" s="359" t="s">
         <v>150</v>
       </c>
-      <c r="L3" s="352"/>
-      <c r="M3" s="351" t="s">
+      <c r="L3" s="360"/>
+      <c r="M3" s="359" t="s">
         <v>151</v>
       </c>
-      <c r="N3" s="353"/>
+      <c r="N3" s="361"/>
     </row>
     <row r="4" spans="1:14" ht="43.5" customHeight="1">
       <c r="A4" s="165" t="s">
         <v>152</v>
       </c>
-      <c r="B4" s="354" t="s">
+      <c r="B4" s="362" t="s">
         <v>153</v>
       </c>
-      <c r="C4" s="355"/>
-      <c r="D4" s="355"/>
-      <c r="E4" s="355"/>
-      <c r="F4" s="355"/>
-      <c r="G4" s="355"/>
-      <c r="H4" s="356"/>
-      <c r="I4" s="357"/>
-      <c r="J4" s="358"/>
-      <c r="K4" s="357"/>
-      <c r="L4" s="358"/>
-      <c r="M4" s="357"/>
-      <c r="N4" s="359"/>
+      <c r="C4" s="363"/>
+      <c r="D4" s="363"/>
+      <c r="E4" s="363"/>
+      <c r="F4" s="363"/>
+      <c r="G4" s="363"/>
+      <c r="H4" s="364"/>
+      <c r="I4" s="365"/>
+      <c r="J4" s="366"/>
+      <c r="K4" s="365"/>
+      <c r="L4" s="366"/>
+      <c r="M4" s="365"/>
+      <c r="N4" s="367"/>
     </row>
     <row r="5" spans="1:14" s="167" customFormat="1" ht="46.5" customHeight="1">
       <c r="A5" s="166">
         <v>1</v>
       </c>
-      <c r="B5" s="362" t="s">
+      <c r="B5" s="333" t="s">
         <v>154</v>
       </c>
-      <c r="C5" s="363"/>
-      <c r="D5" s="363"/>
-      <c r="E5" s="363"/>
-      <c r="F5" s="363"/>
-      <c r="G5" s="363"/>
-      <c r="H5" s="363"/>
-      <c r="I5" s="363"/>
-      <c r="J5" s="363"/>
-      <c r="K5" s="363"/>
-      <c r="L5" s="363"/>
-      <c r="M5" s="363"/>
-      <c r="N5" s="364"/>
+      <c r="C5" s="334"/>
+      <c r="D5" s="334"/>
+      <c r="E5" s="334"/>
+      <c r="F5" s="334"/>
+      <c r="G5" s="334"/>
+      <c r="H5" s="334"/>
+      <c r="I5" s="334"/>
+      <c r="J5" s="334"/>
+      <c r="K5" s="334"/>
+      <c r="L5" s="334"/>
+      <c r="M5" s="334"/>
+      <c r="N5" s="335"/>
     </row>
     <row r="6" spans="1:14" s="167" customFormat="1" ht="39" customHeight="1">
       <c r="A6" s="168">
         <v>2</v>
       </c>
-      <c r="B6" s="365" t="s">
+      <c r="B6" s="336" t="s">
         <v>155</v>
       </c>
-      <c r="C6" s="366"/>
-      <c r="D6" s="366"/>
-      <c r="E6" s="366"/>
-      <c r="F6" s="366"/>
-      <c r="G6" s="366"/>
-      <c r="H6" s="366"/>
-      <c r="I6" s="366"/>
-      <c r="J6" s="366"/>
-      <c r="K6" s="366"/>
-      <c r="L6" s="366"/>
-      <c r="M6" s="366"/>
-      <c r="N6" s="367"/>
+      <c r="C6" s="337"/>
+      <c r="D6" s="337"/>
+      <c r="E6" s="337"/>
+      <c r="F6" s="337"/>
+      <c r="G6" s="337"/>
+      <c r="H6" s="337"/>
+      <c r="I6" s="337"/>
+      <c r="J6" s="337"/>
+      <c r="K6" s="337"/>
+      <c r="L6" s="337"/>
+      <c r="M6" s="337"/>
+      <c r="N6" s="338"/>
     </row>
     <row r="7" spans="1:14" s="167" customFormat="1" ht="21" customHeight="1">
       <c r="A7" s="169" t="s">
         <v>156</v>
       </c>
-      <c r="B7" s="368" t="s">
+      <c r="B7" s="339" t="s">
         <v>157</v>
       </c>
-      <c r="C7" s="369"/>
-      <c r="D7" s="369"/>
-      <c r="E7" s="369"/>
-      <c r="F7" s="369"/>
-      <c r="G7" s="369"/>
-      <c r="H7" s="369"/>
-      <c r="I7" s="369"/>
-      <c r="J7" s="369"/>
-      <c r="K7" s="369"/>
-      <c r="L7" s="369"/>
-      <c r="M7" s="369"/>
-      <c r="N7" s="370"/>
+      <c r="C7" s="340"/>
+      <c r="D7" s="340"/>
+      <c r="E7" s="340"/>
+      <c r="F7" s="340"/>
+      <c r="G7" s="340"/>
+      <c r="H7" s="340"/>
+      <c r="I7" s="340"/>
+      <c r="J7" s="340"/>
+      <c r="K7" s="340"/>
+      <c r="L7" s="340"/>
+      <c r="M7" s="340"/>
+      <c r="N7" s="341"/>
     </row>
     <row r="8" spans="1:14" s="174" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="170"/>
@@ -38848,7 +38848,7 @@
       <c r="N42" s="178"/>
     </row>
     <row r="43" spans="1:14" s="202" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A43" s="371" t="s">
+      <c r="A43" s="342" t="s">
         <v>162</v>
       </c>
       <c r="B43" s="195" t="s">
@@ -38856,81 +38856,95 @@
       </c>
       <c r="C43" s="196"/>
       <c r="D43" s="197"/>
-      <c r="E43" s="374"/>
-      <c r="F43" s="375"/>
-      <c r="G43" s="375"/>
-      <c r="H43" s="375"/>
-      <c r="I43" s="375"/>
-      <c r="J43" s="375"/>
+      <c r="E43" s="345"/>
+      <c r="F43" s="346"/>
+      <c r="G43" s="346"/>
+      <c r="H43" s="346"/>
+      <c r="I43" s="346"/>
+      <c r="J43" s="346"/>
       <c r="K43" s="200"/>
       <c r="L43" s="199"/>
       <c r="M43" s="198"/>
       <c r="N43" s="201"/>
     </row>
     <row r="44" spans="1:14" s="202" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A44" s="372"/>
+      <c r="A44" s="343"/>
       <c r="B44" s="203" t="s">
         <v>163</v>
       </c>
       <c r="C44" s="204"/>
       <c r="D44" s="205"/>
-      <c r="E44" s="376"/>
-      <c r="F44" s="377"/>
-      <c r="G44" s="377"/>
-      <c r="H44" s="377"/>
-      <c r="I44" s="377"/>
-      <c r="J44" s="377"/>
+      <c r="E44" s="347"/>
+      <c r="F44" s="348"/>
+      <c r="G44" s="348"/>
+      <c r="H44" s="348"/>
+      <c r="I44" s="348"/>
+      <c r="J44" s="348"/>
       <c r="K44" s="206"/>
       <c r="L44" s="207"/>
       <c r="M44" s="208"/>
       <c r="N44" s="209"/>
     </row>
     <row r="45" spans="1:14" s="202" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A45" s="372"/>
+      <c r="A45" s="343"/>
       <c r="B45" s="210" t="s">
         <v>164</v>
       </c>
       <c r="C45" s="204"/>
       <c r="D45" s="205"/>
-      <c r="E45" s="378"/>
-      <c r="F45" s="379"/>
-      <c r="G45" s="379"/>
-      <c r="H45" s="379"/>
-      <c r="I45" s="379"/>
-      <c r="J45" s="379"/>
+      <c r="E45" s="349"/>
+      <c r="F45" s="350"/>
+      <c r="G45" s="350"/>
+      <c r="H45" s="350"/>
+      <c r="I45" s="350"/>
+      <c r="J45" s="350"/>
       <c r="K45" s="211"/>
       <c r="L45" s="207"/>
       <c r="M45" s="212"/>
       <c r="N45" s="213"/>
     </row>
     <row r="46" spans="1:14" s="202" customFormat="1" ht="25.5" customHeight="1" thickBot="1">
-      <c r="A46" s="373"/>
+      <c r="A46" s="344"/>
       <c r="B46" s="214" t="s">
         <v>165</v>
       </c>
-      <c r="C46" s="380" t="s">
+      <c r="C46" s="351" t="s">
         <v>166</v>
       </c>
-      <c r="D46" s="381"/>
-      <c r="E46" s="382" t="s">
+      <c r="D46" s="352"/>
+      <c r="E46" s="353" t="s">
         <v>167</v>
       </c>
-      <c r="F46" s="383"/>
-      <c r="G46" s="383"/>
-      <c r="H46" s="383"/>
-      <c r="I46" s="383"/>
-      <c r="J46" s="384"/>
-      <c r="K46" s="360" t="s">
+      <c r="F46" s="354"/>
+      <c r="G46" s="354"/>
+      <c r="H46" s="354"/>
+      <c r="I46" s="354"/>
+      <c r="J46" s="355"/>
+      <c r="K46" s="331" t="s">
         <v>168</v>
       </c>
-      <c r="L46" s="384"/>
-      <c r="M46" s="360" t="s">
+      <c r="L46" s="355"/>
+      <c r="M46" s="331" t="s">
         <v>169</v>
       </c>
-      <c r="N46" s="361"/>
+      <c r="N46" s="332"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="M46:N46"/>
     <mergeCell ref="B5:N5"/>
     <mergeCell ref="B6:N6"/>
@@ -38942,20 +38956,6 @@
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="E46:J46"/>
     <mergeCell ref="K46:L46"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="L2:N2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -38995,29 +38995,29 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="26.25">
-      <c r="A3" s="320" t="s">
+      <c r="A3" s="321" t="s">
         <v>229</v>
       </c>
-      <c r="B3" s="320"/>
-      <c r="C3" s="320"/>
-      <c r="D3" s="320"/>
-      <c r="E3" s="320"/>
-      <c r="F3" s="320"/>
-      <c r="G3" s="320"/>
-      <c r="H3" s="320"/>
-      <c r="I3" s="320"/>
-      <c r="J3" s="320"/>
-      <c r="K3" s="320"/>
-      <c r="L3" s="320"/>
+      <c r="B3" s="321"/>
+      <c r="C3" s="321"/>
+      <c r="D3" s="321"/>
+      <c r="E3" s="321"/>
+      <c r="F3" s="321"/>
+      <c r="G3" s="321"/>
+      <c r="H3" s="321"/>
+      <c r="I3" s="321"/>
+      <c r="J3" s="321"/>
+      <c r="K3" s="321"/>
+      <c r="L3" s="321"/>
     </row>
     <row r="4" spans="1:12" ht="20.100000000000001" customHeight="1">
       <c r="H4" s="56" t="s">
         <v>88</v>
       </c>
-      <c r="I4" s="389">
+      <c r="I4" s="390">
         <v>45390</v>
       </c>
-      <c r="J4" s="389"/>
+      <c r="J4" s="390"/>
       <c r="K4" s="73"/>
       <c r="L4" s="73"/>
     </row>
@@ -39031,12 +39031,12 @@
       <c r="H5" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="I5" s="326" t="s">
+      <c r="I5" s="327" t="s">
         <v>319</v>
       </c>
-      <c r="J5" s="326"/>
-      <c r="K5" s="326"/>
-      <c r="L5" s="326"/>
+      <c r="J5" s="327"/>
+      <c r="K5" s="327"/>
+      <c r="L5" s="327"/>
     </row>
     <row r="6" spans="1:12" ht="20.25" customHeight="1">
       <c r="B6" t="s">
@@ -39045,10 +39045,10 @@
       <c r="H6" s="56" t="s">
         <v>90</v>
       </c>
-      <c r="I6" s="326" t="s">
+      <c r="I6" s="327" t="s">
         <v>235</v>
       </c>
-      <c r="J6" s="326"/>
+      <c r="J6" s="327"/>
       <c r="K6" s="74"/>
       <c r="L6" s="74"/>
     </row>
@@ -39077,32 +39077,32 @@
       <c r="L8" s="13"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1">
-      <c r="J9" s="327" t="s">
+      <c r="J9" s="328" t="s">
         <v>132</v>
       </c>
-      <c r="K9" s="328" t="s">
+      <c r="K9" s="329" t="s">
         <v>140</v>
       </c>
-      <c r="L9" s="329"/>
+      <c r="L9" s="330"/>
     </row>
     <row r="10" spans="1:12">
       <c r="B10" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="323" t="s">
+      <c r="C10" s="324" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="324"/>
-      <c r="E10" s="325"/>
+      <c r="D10" s="325"/>
+      <c r="E10" s="326"/>
       <c r="F10" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="G10" s="323" t="s">
+      <c r="G10" s="324" t="s">
         <v>56</v>
       </c>
-      <c r="H10" s="324"/>
+      <c r="H10" s="325"/>
       <c r="I10" s="13"/>
-      <c r="J10" s="327"/>
+      <c r="J10" s="328"/>
       <c r="K10" s="9" t="s">
         <v>141</v>
       </c>
@@ -39114,14 +39114,14 @@
       <c r="B11" s="221" t="s">
         <v>234</v>
       </c>
-      <c r="C11" s="387" t="s">
+      <c r="C11" s="388" t="s">
         <v>235</v>
       </c>
-      <c r="D11" s="388"/>
-      <c r="E11" s="325"/>
+      <c r="D11" s="389"/>
+      <c r="E11" s="326"/>
       <c r="F11" s="51"/>
-      <c r="G11" s="321"/>
-      <c r="H11" s="322"/>
+      <c r="G11" s="322"/>
+      <c r="H11" s="323"/>
       <c r="I11" s="13"/>
       <c r="J11" s="9"/>
       <c r="K11" s="10"/>
@@ -40461,10 +40461,10 @@
       <c r="L48" s="9"/>
     </row>
     <row r="49" spans="1:12" ht="17.25" customHeight="1">
-      <c r="A49" s="385" t="s">
+      <c r="A49" s="386" t="s">
         <v>392</v>
       </c>
-      <c r="B49" s="386"/>
+      <c r="B49" s="387"/>
       <c r="C49" s="219"/>
       <c r="D49" s="219"/>
       <c r="E49" s="219"/>
@@ -40488,23 +40488,23 @@
     </row>
     <row r="51" spans="1:12" ht="18" customHeight="1"/>
     <row r="52" spans="1:12">
-      <c r="A52" s="328" t="s">
+      <c r="A52" s="329" t="s">
         <v>95</v>
       </c>
-      <c r="B52" s="329"/>
-      <c r="C52" s="328" t="s">
+      <c r="B52" s="330"/>
+      <c r="C52" s="329" t="s">
         <v>93</v>
       </c>
-      <c r="D52" s="329"/>
-      <c r="E52" s="328" t="s">
+      <c r="D52" s="330"/>
+      <c r="E52" s="329" t="s">
         <v>221</v>
       </c>
-      <c r="F52" s="329"/>
-      <c r="G52" s="327" t="s">
+      <c r="F52" s="330"/>
+      <c r="G52" s="328" t="s">
         <v>231</v>
       </c>
-      <c r="H52" s="327"/>
-      <c r="I52" s="327"/>
+      <c r="H52" s="328"/>
+      <c r="I52" s="328"/>
       <c r="J52" s="58" t="s">
         <v>230</v>
       </c>
@@ -40564,17 +40564,22 @@
         <v>88</v>
       </c>
       <c r="F57" s="68"/>
-      <c r="G57" s="317" t="s">
+      <c r="G57" s="318" t="s">
         <v>88</v>
       </c>
-      <c r="H57" s="318"/>
-      <c r="I57" s="319"/>
+      <c r="H57" s="319"/>
+      <c r="I57" s="320"/>
       <c r="J57" s="10" t="s">
         <v>88</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="E52:F52"/>
+    <mergeCell ref="G52:I52"/>
+    <mergeCell ref="G57:I57"/>
     <mergeCell ref="A49:B49"/>
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:L3"/>
@@ -40588,11 +40593,6 @@
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="I4:J4"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="E52:F52"/>
-    <mergeCell ref="G52:I52"/>
-    <mergeCell ref="G57:I57"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="68" orientation="portrait" r:id="rId1"/>
@@ -40633,29 +40633,29 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="26.25">
-      <c r="A3" s="320" t="s">
+      <c r="A3" s="321" t="s">
         <v>229</v>
       </c>
-      <c r="B3" s="320"/>
-      <c r="C3" s="320"/>
-      <c r="D3" s="320"/>
-      <c r="E3" s="320"/>
-      <c r="F3" s="320"/>
-      <c r="G3" s="320"/>
-      <c r="H3" s="320"/>
-      <c r="I3" s="320"/>
-      <c r="J3" s="320"/>
-      <c r="K3" s="320"/>
-      <c r="L3" s="320"/>
+      <c r="B3" s="321"/>
+      <c r="C3" s="321"/>
+      <c r="D3" s="321"/>
+      <c r="E3" s="321"/>
+      <c r="F3" s="321"/>
+      <c r="G3" s="321"/>
+      <c r="H3" s="321"/>
+      <c r="I3" s="321"/>
+      <c r="J3" s="321"/>
+      <c r="K3" s="321"/>
+      <c r="L3" s="321"/>
     </row>
     <row r="4" spans="1:12" ht="20.100000000000001" customHeight="1">
       <c r="H4" s="56" t="s">
         <v>88</v>
       </c>
-      <c r="I4" s="389">
+      <c r="I4" s="390">
         <v>45390</v>
       </c>
-      <c r="J4" s="389"/>
+      <c r="J4" s="390"/>
       <c r="K4" s="73"/>
       <c r="L4" s="73"/>
     </row>
@@ -40669,12 +40669,12 @@
       <c r="H5" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="I5" s="326" t="s">
+      <c r="I5" s="327" t="s">
         <v>319</v>
       </c>
-      <c r="J5" s="326"/>
-      <c r="K5" s="326"/>
-      <c r="L5" s="326"/>
+      <c r="J5" s="327"/>
+      <c r="K5" s="327"/>
+      <c r="L5" s="327"/>
     </row>
     <row r="6" spans="1:12" ht="20.25" customHeight="1">
       <c r="B6" t="s">
@@ -40683,10 +40683,10 @@
       <c r="H6" s="56" t="s">
         <v>90</v>
       </c>
-      <c r="I6" s="326" t="s">
+      <c r="I6" s="327" t="s">
         <v>235</v>
       </c>
-      <c r="J6" s="326"/>
+      <c r="J6" s="327"/>
       <c r="K6" s="74"/>
       <c r="L6" s="74"/>
     </row>
@@ -40715,32 +40715,32 @@
       <c r="L8" s="13"/>
     </row>
     <row r="9" spans="1:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="J9" s="327" t="s">
+      <c r="J9" s="328" t="s">
         <v>132</v>
       </c>
-      <c r="K9" s="328" t="s">
+      <c r="K9" s="329" t="s">
         <v>140</v>
       </c>
-      <c r="L9" s="329"/>
+      <c r="L9" s="330"/>
     </row>
     <row r="10" spans="1:12">
       <c r="B10" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="323" t="s">
+      <c r="C10" s="324" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="324"/>
-      <c r="E10" s="325"/>
+      <c r="D10" s="325"/>
+      <c r="E10" s="326"/>
       <c r="F10" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="G10" s="323" t="s">
+      <c r="G10" s="324" t="s">
         <v>56</v>
       </c>
-      <c r="H10" s="324"/>
+      <c r="H10" s="325"/>
       <c r="I10" s="13"/>
-      <c r="J10" s="327"/>
+      <c r="J10" s="328"/>
       <c r="K10" s="9" t="s">
         <v>141</v>
       </c>
@@ -40752,14 +40752,14 @@
       <c r="B11" s="221" t="s">
         <v>234</v>
       </c>
-      <c r="C11" s="387" t="s">
+      <c r="C11" s="388" t="s">
         <v>235</v>
       </c>
-      <c r="D11" s="388"/>
-      <c r="E11" s="325"/>
+      <c r="D11" s="389"/>
+      <c r="E11" s="326"/>
       <c r="F11" s="51"/>
-      <c r="G11" s="321"/>
-      <c r="H11" s="322"/>
+      <c r="G11" s="322"/>
+      <c r="H11" s="323"/>
       <c r="I11" s="13"/>
       <c r="J11" s="9"/>
       <c r="K11" s="10"/>
@@ -42433,10 +42433,10 @@
       <c r="L57" s="9"/>
     </row>
     <row r="58" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A58" s="390" t="s">
+      <c r="A58" s="391" t="s">
         <v>392</v>
       </c>
-      <c r="B58" s="390"/>
+      <c r="B58" s="391"/>
       <c r="C58" s="67"/>
       <c r="D58" s="222"/>
       <c r="E58" s="219"/>
@@ -42453,23 +42453,23 @@
     </row>
     <row r="59" spans="1:12" ht="21" customHeight="1"/>
     <row r="60" spans="1:12">
-      <c r="A60" s="328" t="s">
+      <c r="A60" s="329" t="s">
         <v>95</v>
       </c>
-      <c r="B60" s="329"/>
-      <c r="C60" s="328" t="s">
+      <c r="B60" s="330"/>
+      <c r="C60" s="329" t="s">
         <v>93</v>
       </c>
-      <c r="D60" s="329"/>
-      <c r="E60" s="328" t="s">
+      <c r="D60" s="330"/>
+      <c r="E60" s="329" t="s">
         <v>221</v>
       </c>
-      <c r="F60" s="329"/>
-      <c r="G60" s="327" t="s">
+      <c r="F60" s="330"/>
+      <c r="G60" s="328" t="s">
         <v>231</v>
       </c>
-      <c r="H60" s="327"/>
-      <c r="I60" s="327"/>
+      <c r="H60" s="328"/>
+      <c r="I60" s="328"/>
       <c r="J60" s="58" t="s">
         <v>230</v>
       </c>
@@ -42529,17 +42529,27 @@
         <v>88</v>
       </c>
       <c r="F65" s="68"/>
-      <c r="G65" s="317" t="s">
+      <c r="G65" s="318" t="s">
         <v>88</v>
       </c>
-      <c r="H65" s="318"/>
-      <c r="I65" s="319"/>
+      <c r="H65" s="319"/>
+      <c r="I65" s="320"/>
       <c r="J65" s="10" t="s">
         <v>88</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="G65:I65"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="C11:D11"/>
@@ -42548,16 +42558,6 @@
     <mergeCell ref="C60:D60"/>
     <mergeCell ref="E60:F60"/>
     <mergeCell ref="G60:I60"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="G10:H10"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="68" orientation="portrait" r:id="rId1"/>

</xml_diff>